<commit_message>
file acces command switched from xlsx to fs in enrichment file
</commit_message>
<xml_diff>
--- a/scrapers/output/Startup_Funding_Data03.xlsx
+++ b/scrapers/output/Startup_Funding_Data03.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Funding Rounds" sheetId="1" r:id="rId1"/>
+    <sheet name="fundingRound" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,16 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G917"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="60.83203125" customWidth="1"/>
-    <col min="7" max="7" width="35.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:H917"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,6 +421,9 @@
       <c r="G1" t="str">
         <v>website</v>
       </c>
+      <c r="H1" t="str">
+        <v>targetEmail</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -451,7 +445,10 @@
         <v>Accel, Formus Capital, Operator Collective</v>
       </c>
       <c r="G2" t="str">
-        <v>sapiom.ai</v>
+        <v>sapiominds.com</v>
+      </c>
+      <c r="H2" t="str">
+        <v>careers@sapiominds.com</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +471,10 @@
         <v/>
       </c>
       <c r="G3" t="str">
-        <v>callbaba.com</v>
+        <v>ba-bamail.com</v>
+      </c>
+      <c r="H3" t="str">
+        <v>careers@ba-bamail.com</v>
       </c>
     </row>
     <row r="4">
@@ -497,7 +497,10 @@
         <v/>
       </c>
       <c r="G4" t="str">
-        <v>quantumtiger.in</v>
+        <v>quantumtigergames.com</v>
+      </c>
+      <c r="H4" t="str">
+        <v>careers@quantumtigergames.com</v>
       </c>
     </row>
     <row r="5">
@@ -520,7 +523,10 @@
         <v>BEENEXT, Eximius Ventures</v>
       </c>
       <c r="G5" t="str">
-        <v>prolearn.app</v>
+        <v>prolearners.lk</v>
+      </c>
+      <c r="H5" t="str">
+        <v>careers@prolearners.lk</v>
       </c>
     </row>
     <row r="6">
@@ -543,7 +549,10 @@
         <v>Amiya Pathak, Asad Khan, Ramakant Sharma</v>
       </c>
       <c r="G6" t="str">
-        <v>xccelera.ai</v>
+        <v>xccelerate.co</v>
+      </c>
+      <c r="H6" t="str">
+        <v>careers@xccelerate.co</v>
       </c>
     </row>
     <row r="7">
@@ -566,7 +575,10 @@
         <v>Antler, DeVC, Nandan Reddy, Sriharsha Majety</v>
       </c>
       <c r="G7" t="str">
-        <v>stance.health</v>
+        <v>stancehealthcare.com</v>
+      </c>
+      <c r="H7" t="str">
+        <v>careers@stancehealthcare.com</v>
       </c>
     </row>
     <row r="8">
@@ -658,7 +670,10 @@
         <v>Eximius Ventures, First Cheque, Info Edge ventures, Misfits</v>
       </c>
       <c r="G11" t="str">
-        <v>30sundays.club</v>
+        <v>sundaysocial.tv</v>
+      </c>
+      <c r="H11" t="str">
+        <v>careers@sundaysocial.tv</v>
       </c>
     </row>
     <row r="12">
@@ -750,7 +765,10 @@
         <v>Pavestone Capital</v>
       </c>
       <c r="G15" t="str">
-        <v>tsavoritesi.com/#</v>
+        <v>tsavorite.com</v>
+      </c>
+      <c r="H15" t="str">
+        <v>careers@tsavorite.com</v>
       </c>
     </row>
     <row r="16">
@@ -775,6 +793,9 @@
       <c r="G16" t="str">
         <v>umagine.co.in</v>
       </c>
+      <c r="H16" t="str">
+        <v>careers@umagine.co.in</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -865,7 +886,10 @@
         <v>77 Capital, Amplify, Bharat Founders Fund, GSF, Powerhouse Ventures, Untitled Ventures</v>
       </c>
       <c r="G20" t="str">
-        <v>carepay.money</v>
+        <v>carepayment.com</v>
+      </c>
+      <c r="H20" t="str">
+        <v>careers@carepayment.com</v>
       </c>
     </row>
     <row r="21">
@@ -934,7 +958,10 @@
         <v>Research Innovation Incubation Design Laboratory</v>
       </c>
       <c r="G23" t="str">
-        <v>dcverse.in</v>
+        <v>d2cverse.club</v>
+      </c>
+      <c r="H23" t="str">
+        <v>careers@d2cverse.club</v>
       </c>
     </row>
     <row r="24">
@@ -957,7 +984,10 @@
         <v/>
       </c>
       <c r="G24" t="str">
-        <v>nirmaan360.com</v>
+        <v>bdbangurendowment.com</v>
+      </c>
+      <c r="H24" t="str">
+        <v>careers@bdbangurendowment.com</v>
       </c>
     </row>
     <row r="25">
@@ -980,7 +1010,10 @@
         <v>AWS Space Accelerator</v>
       </c>
       <c r="G25" t="str">
-        <v>taramandal.co.in</v>
+        <v>taramandala.org</v>
+      </c>
+      <c r="H25" t="str">
+        <v>careers@taramandala.org</v>
       </c>
     </row>
     <row r="26">
@@ -1026,7 +1059,10 @@
         <v>Aakash Chaudhry, Abhay Agarwal, Action Tesa, Arun Jain, Burman Family Holdings, Devesh Sachdev, Lightspeed India Partners, MMG Group Family Office, MS Dhoni Family Office, Navin Jain, NB Ventures, Panthera Peak Ventures, Paramark Ventures, Pravin Jain, Pravin Jain, Purrshottam Bhaggeria, Ritesh Agarwal, Shantanu Agarwal, Vishal Dhupar</v>
       </c>
       <c r="G27" t="str">
-        <v>centricity.co.in</v>
+        <v>centricity.org</v>
+      </c>
+      <c r="H27" t="str">
+        <v>careers@centricity.org</v>
       </c>
     </row>
     <row r="28">
@@ -1049,7 +1085,10 @@
         <v>Microsoft for Startups</v>
       </c>
       <c r="G28" t="str">
-        <v>hydromind.in</v>
+        <v>hydromindsurf.com</v>
+      </c>
+      <c r="H28" t="str">
+        <v>careers@hydromindsurf.com</v>
       </c>
     </row>
     <row r="29">
@@ -1072,7 +1111,10 @@
         <v>Chinmaya Sharma, Dragon Capital, Goodwater Capital, Java Capital, Mayank Kumar, Metaplanet, Original Capital, Pratyush Prasanna, Soma Capital, Sudhanshu Raheja, Super Capital VC, Taurus Ventures, Tremis Capital, Y Combinator</v>
       </c>
       <c r="G29" t="str">
-        <v>tube11.in</v>
+        <v>betteropinions.in</v>
+      </c>
+      <c r="H29" t="str">
+        <v>careers@betteropinions.in</v>
       </c>
     </row>
     <row r="30">
@@ -1097,6 +1139,9 @@
       <c r="G30" t="str">
         <v>daolens.com</v>
       </c>
+      <c r="H30" t="str">
+        <v>careers@daolens.com</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1120,6 +1165,9 @@
       <c r="G31" t="str">
         <v>chhotastock.com</v>
       </c>
+      <c r="H31" t="str">
+        <v>careers@chhotastock.com</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1143,6 +1191,9 @@
       <c r="G32" t="str">
         <v>nesobrands.com</v>
       </c>
+      <c r="H32" t="str">
+        <v>careers@nesobrands.com</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1166,6 +1217,9 @@
       <c r="G33" t="str">
         <v>koinbasket.com</v>
       </c>
+      <c r="H33" t="str">
+        <v>careers@koinbasket.com</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1187,7 +1241,10 @@
         <v/>
       </c>
       <c r="G34" t="str">
-        <v>konectu.in</v>
+        <v>konectus.org</v>
+      </c>
+      <c r="H34" t="str">
+        <v>careers@konectus.org</v>
       </c>
     </row>
     <row r="35">
@@ -1212,6 +1269,9 @@
       <c r="G35" t="str">
         <v>fanztar.com</v>
       </c>
+      <c r="H35" t="str">
+        <v>careers@fanztar.com</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1235,6 +1295,9 @@
       <c r="G36" t="str">
         <v>scrollify.in</v>
       </c>
+      <c r="H36" t="str">
+        <v>careers@scrollify.in</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1256,7 +1319,10 @@
         <v>Alkemi Growth Capital, Shree Vasu Logistics Limited</v>
       </c>
       <c r="G37" t="str">
-        <v>alphadroid.io</v>
+        <v>alphadroid.com</v>
+      </c>
+      <c r="H37" t="str">
+        <v>careers@alphadroid.com</v>
       </c>
     </row>
     <row r="38">
@@ -1279,7 +1345,10 @@
         <v>100X.VC</v>
       </c>
       <c r="G38" t="str">
-        <v>rethought.in</v>
+        <v>re-thought.com</v>
+      </c>
+      <c r="H38" t="str">
+        <v>careers@re-thought.com</v>
       </c>
     </row>
     <row r="39">
@@ -1370,6 +1439,9 @@
       <c r="G42" t="str">
         <v>sudofoods.com</v>
       </c>
+      <c r="H42" t="str">
+        <v>careers@sudofoods.com</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -1414,7 +1486,10 @@
         <v>100Unicorns, Alphatron Capital, Anand Chandrasekaran, Ashish Gupta, Aureolis Ventures, Dholakia Ventures, Dovetail, Inventus Capital Partners, Jayan Ramankutty, Kalyan Krishnamurthy, KL Rahul, Kwaish Ventures, Nandi Vardhan Mehta, NB Ventures, Rahul Seth, Raju Reddy, RTP Global, Shivakumar Ganesan, Srinivas Anumolu, Sujeet Kumar, Sundi Natarajan, SVQUAD, Turbostart, Twin Ventures, Upsparks</v>
       </c>
       <c r="G44" t="str">
-        <v>flamapp.com</v>
+        <v>flamingtext.com</v>
+      </c>
+      <c r="H44" t="str">
+        <v>careers@flamingtext.com</v>
       </c>
     </row>
     <row r="45">
@@ -1439,6 +1514,9 @@
       <c r="G45" t="str">
         <v>upswing.one</v>
       </c>
+      <c r="H45" t="str">
+        <v>careers@upswing.one</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -1462,6 +1540,9 @@
       <c r="G46" t="str">
         <v>truefoundry.com</v>
       </c>
+      <c r="H46" t="str">
+        <v>careers@truefoundry.com</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -1485,6 +1566,9 @@
       <c r="G47" t="str">
         <v>zippmat.com</v>
       </c>
+      <c r="H47" t="str">
+        <v>careers@zippmat.com</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1506,7 +1590,10 @@
         <v>Alliance DAO, Anagram, Anatoly Yakovenko, Balaji Srinivasan, Peak XV Partners, Raj Gokal, Sandeep Nailwal</v>
       </c>
       <c r="G48" t="str">
-        <v>0xppl.com</v>
+        <v>xppublicitarios.com</v>
+      </c>
+      <c r="H48" t="str">
+        <v>careers@xppublicitarios.com</v>
       </c>
     </row>
     <row r="49">
@@ -1531,6 +1618,9 @@
       <c r="G49" t="str">
         <v>sundaydesign.in</v>
       </c>
+      <c r="H49" t="str">
+        <v>careers@sundaydesign.in</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -1552,7 +1642,10 @@
         <v>Aniket Jindal, Arcanum Capital, Graviton Web3 Accelerator, Lancer Capital, Prabhakar Reddy, Tushar Aggarwal, Woodstock Fund</v>
       </c>
       <c r="G50" t="str">
-        <v>wall.app</v>
+        <v>wallethub.com</v>
+      </c>
+      <c r="H50" t="str">
+        <v>careers@wallethub.com</v>
       </c>
     </row>
     <row r="51">
@@ -1575,7 +1668,10 @@
         <v/>
       </c>
       <c r="G51" t="str">
-        <v>boondfragrances.com</v>
+        <v>boondockerswelcome.com</v>
+      </c>
+      <c r="H51" t="str">
+        <v>careers@boondockerswelcome.com</v>
       </c>
     </row>
     <row r="52">
@@ -1600,6 +1696,9 @@
       <c r="G52" t="str">
         <v>tassets.in</v>
       </c>
+      <c r="H52" t="str">
+        <v>careers@tassets.in</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -1646,6 +1745,9 @@
       <c r="G54" t="str">
         <v>insightgig.com</v>
       </c>
+      <c r="H54" t="str">
+        <v>careers@insightgig.com</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -1690,7 +1792,10 @@
         <v>PedalStart</v>
       </c>
       <c r="G56" t="str">
-        <v>shoegr.com</v>
+        <v>shoegrab.com.au</v>
+      </c>
+      <c r="H56" t="str">
+        <v>careers@shoegrab.com.au</v>
       </c>
     </row>
     <row r="57">
@@ -1715,6 +1820,9 @@
       <c r="G57" t="str">
         <v>blueenergymotors.com</v>
       </c>
+      <c r="H57" t="str">
+        <v>careers@blueenergymotors.com</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -1759,7 +1867,10 @@
         <v>Athera Venture Partners</v>
       </c>
       <c r="G59" t="str">
-        <v>fanstan.co</v>
+        <v>chinabrandinggroup.com</v>
+      </c>
+      <c r="H59" t="str">
+        <v>careers@chinabrandinggroup.com</v>
       </c>
     </row>
     <row r="60">
@@ -1784,6 +1895,9 @@
       <c r="G60" t="str">
         <v>rapidaivision.com</v>
       </c>
+      <c r="H60" t="str">
+        <v>careers@rapidaivision.com</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -1830,6 +1944,9 @@
       <c r="G62" t="str">
         <v>easyaspataal.com</v>
       </c>
+      <c r="H62" t="str">
+        <v>careers@easyaspataal.com</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -1853,6 +1970,9 @@
       <c r="G63" t="str">
         <v>instrucko.com</v>
       </c>
+      <c r="H63" t="str">
+        <v>careers@instrucko.com</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -1876,6 +1996,9 @@
       <c r="G64" t="str">
         <v>bandhoo.com</v>
       </c>
+      <c r="H64" t="str">
+        <v>careers@bandhoo.com</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -1899,6 +2022,9 @@
       <c r="G65" t="str">
         <v>edukemy.com</v>
       </c>
+      <c r="H65" t="str">
+        <v>careers@edukemy.com</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -1922,6 +2048,9 @@
       <c r="G66" t="str">
         <v>thechefkart.com</v>
       </c>
+      <c r="H66" t="str">
+        <v>careers@thechefkart.com</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -1968,6 +2097,9 @@
       <c r="G68" t="str">
         <v>mysutradhar.com</v>
       </c>
+      <c r="H68" t="str">
+        <v>careers@mysutradhar.com</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -1991,6 +2123,9 @@
       <c r="G69" t="str">
         <v>buyofuel.com</v>
       </c>
+      <c r="H69" t="str">
+        <v>careers@buyofuel.com</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2037,6 +2172,9 @@
       <c r="G71" t="str">
         <v>flomobility.com</v>
       </c>
+      <c r="H71" t="str">
+        <v>careers@flomobility.com</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2060,6 +2198,9 @@
       <c r="G72" t="str">
         <v>verdantimpact.com</v>
       </c>
+      <c r="H72" t="str">
+        <v>careers@verdantimpact.com</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -2106,6 +2247,9 @@
       <c r="G74" t="str">
         <v>vsmani.com</v>
       </c>
+      <c r="H74" t="str">
+        <v>careers@vsmani.com</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -2129,6 +2273,9 @@
       <c r="G75" t="str">
         <v>growpital.com</v>
       </c>
+      <c r="H75" t="str">
+        <v>careers@growpital.com</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -2150,7 +2297,10 @@
         <v>IAN Fund</v>
       </c>
       <c r="G76" t="str">
-        <v>rymo.in</v>
+        <v>rymopestcontrol.com</v>
+      </c>
+      <c r="H76" t="str">
+        <v>careers@rymopestcontrol.com</v>
       </c>
     </row>
     <row r="77">
@@ -2173,7 +2323,10 @@
         <v>Alto Partners, Analog Partners, Anjali Bansal, Atin Kukreja, Boon Hwee Koh, Cercano Management, Citi, East Ventures, Endiya Partners, K3 Ventures, KDV Capital, MassMutual Ventures, Mission Holdings, MMV Europe &amp; Asia-Pacific, Nyca Partners, Patrick Walujo, Sahra Growth Capital, Sujeet Kumar, Vulcan Capital</v>
       </c>
       <c r="G77" t="str">
-        <v>qapita.com</v>
+        <v>qapital.com</v>
+      </c>
+      <c r="H77" t="str">
+        <v>careers@qapital.com</v>
       </c>
     </row>
     <row r="78">
@@ -2219,7 +2372,10 @@
         <v>Abhishek Nag, Ajit Isaac, Ghanshyam Dass, Global Founders Capital, Rohit Kale, Toshan Tamhane</v>
       </c>
       <c r="G79" t="str">
-        <v>thecareerlabs.com</v>
+        <v>careerlabs.net</v>
+      </c>
+      <c r="H79" t="str">
+        <v>careers@careerlabs.net</v>
       </c>
     </row>
     <row r="80">
@@ -2242,7 +2398,10 @@
         <v>ah! Ventures, Ameet Desai, Campus Fund, Dilesh Gathani, Gruhas, Marwari Angels, Rajveer Ranawat, Shireen Rangaswamy, Sin Growth Partners</v>
       </c>
       <c r="G80" t="str">
-        <v>parksmart.in</v>
+        <v>parksmart.ca</v>
+      </c>
+      <c r="H80" t="str">
+        <v>careers@parksmart.ca</v>
       </c>
     </row>
     <row r="81">
@@ -2267,6 +2426,9 @@
       <c r="G81" t="str">
         <v>dvarasmartgold.com</v>
       </c>
+      <c r="H81" t="str">
+        <v>careers@dvarasmartgold.com</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -2290,6 +2452,9 @@
       <c r="G82" t="str">
         <v>smartrestroom.in</v>
       </c>
+      <c r="H82" t="str">
+        <v>careers@smartrestroom.in</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -2313,6 +2478,9 @@
       <c r="G83" t="str">
         <v>zingbus.com</v>
       </c>
+      <c r="H83" t="str">
+        <v>careers@zingbus.com</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -2336,6 +2504,9 @@
       <c r="G84" t="str">
         <v>smowcode.com</v>
       </c>
+      <c r="H84" t="str">
+        <v>careers@smowcode.com</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -2357,7 +2528,10 @@
         <v>Rainmatter</v>
       </c>
       <c r="G85" t="str">
-        <v>fold.money</v>
+        <v>fold3.com</v>
+      </c>
+      <c r="H85" t="str">
+        <v>careers@fold3.com</v>
       </c>
     </row>
     <row r="86">
@@ -2380,7 +2554,10 @@
         <v>Disha Shah, Encubay Angel Network, Faad Network, Niloufer Irani, Pratibha Wilson, Tyke</v>
       </c>
       <c r="G86" t="str">
-        <v>skyber.io</v>
+        <v>skyberry.me</v>
+      </c>
+      <c r="H86" t="str">
+        <v>careers@skyberry.me</v>
       </c>
     </row>
     <row r="87">
@@ -2403,7 +2580,10 @@
         <v/>
       </c>
       <c r="G87" t="str">
-        <v>maatri.in</v>
+        <v>maatris.net</v>
+      </c>
+      <c r="H87" t="str">
+        <v>careers@maatris.net</v>
       </c>
     </row>
     <row r="88">
@@ -2451,6 +2631,9 @@
       <c r="G89" t="str">
         <v>thedrivesales.com</v>
       </c>
+      <c r="H89" t="str">
+        <v>careers@thedrivesales.com</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -2497,6 +2680,9 @@
       <c r="G91" t="str">
         <v>edgeneural.ai</v>
       </c>
+      <c r="H91" t="str">
+        <v>careers@edgeneural.ai</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -2520,6 +2706,9 @@
       <c r="G92" t="str">
         <v>plugzmart.com</v>
       </c>
+      <c r="H92" t="str">
+        <v>careers@plugzmart.com</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -2543,6 +2732,9 @@
       <c r="G93" t="str">
         <v>topbeat.in</v>
       </c>
+      <c r="H93" t="str">
+        <v>careers@topbeat.in</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -2564,7 +2756,10 @@
         <v>Amit Singhal, ANIC-ARISE, Anil Chalamalasetty, BlackRock, Department for Promotion of Industry and Internal Trade (DPIIT), GIC, Graph Ventures, LNM India Internet Ventures, MABS, Mahesh Kolli, Mukesh Bansal, Neeraj Arora, Sherpalo Ventures, Solar Industries India, Sutton Capital, Temasek Holdings, Vedanshu Investments, Wami Capital, Waverly, WorldQuant Ventures LLC</v>
       </c>
       <c r="G94" t="str">
-        <v>skyroot.in</v>
+        <v>skyrootshealing.com</v>
+      </c>
+      <c r="H94" t="str">
+        <v>careers@skyrootshealing.com</v>
       </c>
     </row>
     <row r="95">
@@ -2589,6 +2784,9 @@
       <c r="G95" t="str">
         <v>mogiio.com</v>
       </c>
+      <c r="H95" t="str">
+        <v>careers@mogiio.com</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -2610,7 +2808,10 @@
         <v>Balaji Vaidyanathan, Paurush Sonkar, Sandeep Shetty, WEH Ventures</v>
       </c>
       <c r="G96" t="str">
-        <v>Sustvest.com</v>
+        <v>sustvest.com</v>
+      </c>
+      <c r="H96" t="str">
+        <v>careers@sustvest.com</v>
       </c>
     </row>
     <row r="97">
@@ -2635,6 +2836,9 @@
       <c r="G97" t="str">
         <v>wevois.com</v>
       </c>
+      <c r="H97" t="str">
+        <v>careers@wevois.com</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -2656,7 +2860,10 @@
         <v>BlueOrchard Finance S A, British International Investment, Macquarie Capital, Mumbai Angels, Sprint Vc, Venture Catalysts</v>
       </c>
       <c r="G98" t="str">
-        <v>chargezone.co</v>
+        <v>chargezone.com</v>
+      </c>
+      <c r="H98" t="str">
+        <v>careers@chargezone.com</v>
       </c>
     </row>
     <row r="99">
@@ -2681,6 +2888,9 @@
       <c r="G99" t="str">
         <v>securden.com</v>
       </c>
+      <c r="H99" t="str">
+        <v>careers@securden.com</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -2704,6 +2914,9 @@
       <c r="G100" t="str">
         <v>aadar.co</v>
       </c>
+      <c r="H100" t="str">
+        <v>careers@aadar.co</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -2725,7 +2938,10 @@
         <v>Omnivore</v>
       </c>
       <c r="G101" t="str">
-        <v>agri10x.com</v>
+        <v>agrixpert.com</v>
+      </c>
+      <c r="H101" t="str">
+        <v>careers@agrixpert.com</v>
       </c>
     </row>
     <row r="102">
@@ -2750,6 +2966,9 @@
       <c r="G102" t="str">
         <v>jobsquare.com</v>
       </c>
+      <c r="H102" t="str">
+        <v>careers@jobsquare.com</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -2794,7 +3013,10 @@
         <v>Mistry Ventures, Prime Venture Partners, SIDBI</v>
       </c>
       <c r="G104" t="str">
-        <v>momshome.in</v>
+        <v>momshomecare.com</v>
+      </c>
+      <c r="H104" t="str">
+        <v>careers@momshomecare.com</v>
       </c>
     </row>
     <row r="105">
@@ -2817,7 +3039,10 @@
         <v>AngelList India, Anil Bhansali, Brigade Real Estate Accelerator Program (REAP), Corvus Ventures, Forward Slash Capital, Guptaji invests, LetsVenture, Sandeep Kapoor, Sweta Rau</v>
       </c>
       <c r="G105" t="str">
-        <v>exprs.com</v>
+        <v>expr3ss.com</v>
+      </c>
+      <c r="H105" t="str">
+        <v>careers@expr3ss.com</v>
       </c>
     </row>
     <row r="106">
@@ -2840,7 +3065,10 @@
         <v>IIT Mandi Catalyst</v>
       </c>
       <c r="G106" t="str">
-        <v>biofimed.com</v>
+        <v>biofieldtuning.com</v>
+      </c>
+      <c r="H106" t="str">
+        <v>careers@biofieldtuning.com</v>
       </c>
     </row>
     <row r="107">
@@ -2865,6 +3093,9 @@
       <c r="G107" t="str">
         <v>nowpurchase.com</v>
       </c>
+      <c r="H107" t="str">
+        <v>careers@nowpurchase.com</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -2888,6 +3119,9 @@
       <c r="G108" t="str">
         <v>startoonlabs.com</v>
       </c>
+      <c r="H108" t="str">
+        <v>careers@startoonlabs.com</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -2909,7 +3143,10 @@
         <v>ICICI Bank, Orios Venture Partners</v>
       </c>
       <c r="G109" t="str">
-        <v>bizzo.in</v>
+        <v>bizzoffers.com</v>
+      </c>
+      <c r="H109" t="str">
+        <v>careers@bizzoffers.com</v>
       </c>
     </row>
     <row r="110">
@@ -2934,6 +3171,9 @@
       <c r="G110" t="str">
         <v>xpedize.com</v>
       </c>
+      <c r="H110" t="str">
+        <v>careers@xpedize.com</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -2955,7 +3195,10 @@
         <v>India Quotient, Mayfield Fund, Shunwei Capital</v>
       </c>
       <c r="G111" t="str">
-        <v>upwards.in</v>
+        <v>upward.org</v>
+      </c>
+      <c r="H111" t="str">
+        <v>careers@upward.org</v>
       </c>
     </row>
     <row r="112">
@@ -2978,7 +3221,10 @@
         <v>Arali Ventures, Farvatn Venture, Forward Slash Capital, marquee angels, Stratel</v>
       </c>
       <c r="G112" t="str">
-        <v>oivi.co</v>
+        <v>oiv.int</v>
+      </c>
+      <c r="H112" t="str">
+        <v>careers@oiv.int</v>
       </c>
     </row>
     <row r="113">
@@ -3001,7 +3247,10 @@
         <v>India Quotient, Kstart, Marwah Sports, Mayur Desai, Paula Mariwala, Pranav Marwah, RB Investments Pte. Ltd.</v>
       </c>
       <c r="G113" t="str">
-        <v>squareoffnow.com</v>
+        <v>squareoff.in</v>
+      </c>
+      <c r="H113" t="str">
+        <v>careers@squareoff.in</v>
       </c>
     </row>
     <row r="114">
@@ -3024,7 +3273,10 @@
         <v>Rebalance, Roots Ventures</v>
       </c>
       <c r="G114" t="str">
-        <v>plantpower.fit</v>
+        <v>plantpoweredkidneys.com</v>
+      </c>
+      <c r="H114" t="str">
+        <v>careers@plantpoweredkidneys.com</v>
       </c>
     </row>
     <row r="115">
@@ -3049,6 +3301,9 @@
       <c r="G115" t="str">
         <v>workex.jobs</v>
       </c>
+      <c r="H115" t="str">
+        <v>careers@workex.jobs</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -3070,7 +3325,10 @@
         <v>Capital A</v>
       </c>
       <c r="G116" t="str">
-        <v>roado.co.in</v>
+        <v>roadoftheking.com</v>
+      </c>
+      <c r="H116" t="str">
+        <v>careers@roadoftheking.com</v>
       </c>
     </row>
     <row r="117">
@@ -3093,7 +3351,10 @@
         <v>Inflection Point Ventures, SucSEED Venture Partners, Sumpoorna</v>
       </c>
       <c r="G117" t="str">
-        <v>sportido.com</v>
+        <v>sport-idol.com</v>
+      </c>
+      <c r="H117" t="str">
+        <v>careers@sport-idol.com</v>
       </c>
     </row>
     <row r="118">
@@ -3118,6 +3379,9 @@
       <c r="G118" t="str">
         <v>benow.in</v>
       </c>
+      <c r="H118" t="str">
+        <v>careers@benow.in</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -3141,6 +3405,9 @@
       <c r="G119" t="str">
         <v>joinsuperset.com</v>
       </c>
+      <c r="H119" t="str">
+        <v>careers@joinsuperset.com</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -3185,7 +3452,10 @@
         <v>IIMK Live</v>
       </c>
       <c r="G121" t="str">
-        <v>qual5.com</v>
+        <v>qualindia.in</v>
+      </c>
+      <c r="H121" t="str">
+        <v>careers@qualindia.in</v>
       </c>
     </row>
     <row r="122">
@@ -3210,6 +3480,9 @@
       <c r="G122" t="str">
         <v>advisorymandi.com</v>
       </c>
+      <c r="H122" t="str">
+        <v>careers@advisorymandi.com</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -3233,6 +3506,9 @@
       <c r="G123" t="str">
         <v>nutrimoo.com</v>
       </c>
+      <c r="H123" t="str">
+        <v>careers@nutrimoo.com</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -3254,7 +3530,10 @@
         <v>Farooq Adam, First Cheque, India Quotient</v>
       </c>
       <c r="G124" t="str">
-        <v>firstu.in</v>
+        <v>firstunitedbank.com</v>
+      </c>
+      <c r="H124" t="str">
+        <v>careers@firstunitedbank.com</v>
       </c>
     </row>
     <row r="125">
@@ -3279,6 +3558,9 @@
       <c r="G125" t="str">
         <v>cult.fit</v>
       </c>
+      <c r="H125" t="str">
+        <v>careers@cult.fit</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -3302,6 +3584,9 @@
       <c r="G126" t="str">
         <v>roomsoom.com</v>
       </c>
+      <c r="H126" t="str">
+        <v>careers@roomsoom.com</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -3325,6 +3610,9 @@
       <c r="G127" t="str">
         <v>intangles.ai</v>
       </c>
+      <c r="H127" t="str">
+        <v>careers@intangles.ai</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -3348,6 +3636,9 @@
       <c r="G128" t="str">
         <v>jarshsafety.com</v>
       </c>
+      <c r="H128" t="str">
+        <v>careers@jarshsafety.com</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -3371,6 +3662,9 @@
       <c r="G129" t="str">
         <v>frenchcrown.com</v>
       </c>
+      <c r="H129" t="str">
+        <v>careers@frenchcrown.com</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -3394,6 +3688,9 @@
       <c r="G130" t="str">
         <v>coutloot.com</v>
       </c>
+      <c r="H130" t="str">
+        <v>careers@coutloot.com</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -3415,7 +3712,10 @@
         <v>Kunal Shah, Pravin Gandhi, Sandeep Tandon, Smart Start Fund, Vijay Shekhar Sharma, Vishal Gondal</v>
       </c>
       <c r="G131" t="str">
-        <v>remitr.com</v>
+        <v>remithq.com</v>
+      </c>
+      <c r="H131" t="str">
+        <v>careers@remithq.com</v>
       </c>
     </row>
     <row r="132">
@@ -3440,6 +3740,9 @@
       <c r="G132" t="str">
         <v>onmyowntechnology.com</v>
       </c>
+      <c r="H132" t="str">
+        <v>careers@onmyowntechnology.com</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -3463,6 +3766,9 @@
       <c r="G133" t="str">
         <v>tightthenut.com</v>
       </c>
+      <c r="H133" t="str">
+        <v>careers@tightthenut.com</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -3484,7 +3790,10 @@
         <v>Brand Capital</v>
       </c>
       <c r="G134" t="str">
-        <v>gopling.com</v>
+        <v>plinga.com</v>
+      </c>
+      <c r="H134" t="str">
+        <v>careers@plinga.com</v>
       </c>
     </row>
     <row r="135">
@@ -3507,7 +3816,10 @@
         <v>Athamus Ventures</v>
       </c>
       <c r="G135" t="str">
-        <v>refabd.com</v>
+        <v>refabdiaries.com</v>
+      </c>
+      <c r="H135" t="str">
+        <v>careers@refabdiaries.com</v>
       </c>
     </row>
     <row r="136">
@@ -3532,6 +3844,9 @@
       <c r="G136" t="str">
         <v>moovlee.com</v>
       </c>
+      <c r="H136" t="str">
+        <v>careers@moovlee.com</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
@@ -3601,6 +3916,9 @@
       <c r="G139" t="str">
         <v>squadstack.com</v>
       </c>
+      <c r="H139" t="str">
+        <v>careers@squadstack.com</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
@@ -3622,7 +3940,10 @@
         <v>India Quotient</v>
       </c>
       <c r="G140" t="str">
-        <v>rbus.in</v>
+        <v>rbusd.org</v>
+      </c>
+      <c r="H140" t="str">
+        <v>careers@rbusd.org</v>
       </c>
     </row>
     <row r="141">
@@ -3647,6 +3968,9 @@
       <c r="G141" t="str">
         <v>townrush.in</v>
       </c>
+      <c r="H141" t="str">
+        <v>careers@townrush.in</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -3668,7 +3992,10 @@
         <v/>
       </c>
       <c r="G142" t="str">
-        <v>zebi.io</v>
+        <v>zebit.com</v>
+      </c>
+      <c r="H142" t="str">
+        <v>careers@zebit.com</v>
       </c>
     </row>
     <row r="143">
@@ -3691,7 +4018,10 @@
         <v>3one4 Capital, Endiya Partners, Gravity Holdings, iLabs Capital, JG Digital Equity Ventures, Lightspeed India Partners, Microsoft, Peak XV Partners, Salesforce Ventures, SCB 10X, Sequoia Capital, StartupXseed Ventures, State Bank of India, TCV, Teachers’ Venture Growth, Tracxn labs</v>
       </c>
       <c r="G143" t="str">
-        <v>darwinbox.com</v>
+        <v>darwinbox.in</v>
+      </c>
+      <c r="H143" t="str">
+        <v>careers@darwinbox.in</v>
       </c>
     </row>
     <row r="144">
@@ -3714,7 +4044,10 @@
         <v>Kae Capital, Mumbai Angels, White Unicorn Ventures</v>
       </c>
       <c r="G144" t="str">
-        <v>azuro.in</v>
+        <v>azuro-incendie.fr</v>
+      </c>
+      <c r="H144" t="str">
+        <v>careers@azuro-incendie.fr</v>
       </c>
     </row>
     <row r="145">
@@ -3739,6 +4072,9 @@
       <c r="G145" t="str">
         <v>amelioratebiotech.com</v>
       </c>
+      <c r="H145" t="str">
+        <v>careers@amelioratebiotech.com</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -3783,7 +4119,10 @@
         <v>Calcutta Angels</v>
       </c>
       <c r="G147" t="str">
-        <v>zeroinfy.com</v>
+        <v>zeroinfy.in</v>
+      </c>
+      <c r="H147" t="str">
+        <v>careers@zeroinfy.in</v>
       </c>
     </row>
     <row r="148">
@@ -3808,6 +4147,9 @@
       <c r="G148" t="str">
         <v>pharmarack.com</v>
       </c>
+      <c r="H148" t="str">
+        <v>careers@pharmarack.com</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -3831,6 +4173,9 @@
       <c r="G149" t="str">
         <v>hashtaag.com</v>
       </c>
+      <c r="H149" t="str">
+        <v>careers@hashtaag.com</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -3898,7 +4243,10 @@
         <v>Ankit Gupta, Ankit Gupta, Puneet Motihar</v>
       </c>
       <c r="G152" t="str">
-        <v>ithaka.travel</v>
+        <v>ithaka.org</v>
+      </c>
+      <c r="H152" t="str">
+        <v>careers@ithaka.org</v>
       </c>
     </row>
     <row r="153">
@@ -3923,6 +4271,9 @@
       <c r="G153" t="str">
         <v>bigfishventures.in</v>
       </c>
+      <c r="H153" t="str">
+        <v>careers@bigfishventures.in</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -3967,7 +4318,10 @@
         <v>IIMK Live</v>
       </c>
       <c r="G155" t="str">
-        <v>corevalleys.com</v>
+        <v>corevalleysherbals.in</v>
+      </c>
+      <c r="H155" t="str">
+        <v>careers@corevalleysherbals.in</v>
       </c>
     </row>
     <row r="156">
@@ -3990,7 +4344,10 @@
         <v>HDFC Bank, HDFC Standard Life Insurance</v>
       </c>
       <c r="G156" t="str">
-        <v>xanadu.in</v>
+        <v>xanadurealestate.com</v>
+      </c>
+      <c r="H156" t="str">
+        <v>careers@xanadurealestate.com</v>
       </c>
     </row>
     <row r="157">
@@ -4015,6 +4372,9 @@
       <c r="G157" t="str">
         <v>urbancompany.com</v>
       </c>
+      <c r="H157" t="str">
+        <v>careers@urbancompany.com</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -4038,6 +4398,9 @@
       <c r="G158" t="str">
         <v>etherealmachines.com</v>
       </c>
+      <c r="H158" t="str">
+        <v>careers@etherealmachines.com</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
@@ -4059,7 +4422,10 @@
         <v>Harvinder Singh Bhatia</v>
       </c>
       <c r="G159" t="str">
-        <v>neuronme.com</v>
+        <v>neuronation.com</v>
+      </c>
+      <c r="H159" t="str">
+        <v>careers@neuronation.com</v>
       </c>
     </row>
     <row r="160">
@@ -4082,7 +4448,10 @@
         <v>IIM Calcutta Innovation Park</v>
       </c>
       <c r="G160" t="str">
-        <v>medi360.in</v>
+        <v>mediafire.com</v>
+      </c>
+      <c r="H160" t="str">
+        <v>careers@mediafire.com</v>
       </c>
     </row>
     <row r="161">
@@ -4107,6 +4476,9 @@
       <c r="G161" t="str">
         <v>healthians.com</v>
       </c>
+      <c r="H161" t="str">
+        <v>careers@healthians.com</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -4130,6 +4502,9 @@
       <c r="G162" t="str">
         <v>impactguru.com</v>
       </c>
+      <c r="H162" t="str">
+        <v>careers@impactguru.com</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
@@ -4151,7 +4526,10 @@
         <v>Kstart</v>
       </c>
       <c r="G163" t="str">
-        <v>indee.tv</v>
+        <v>indeed.com</v>
+      </c>
+      <c r="H163" t="str">
+        <v>careers@indeed.com</v>
       </c>
     </row>
     <row r="164">
@@ -4174,7 +4552,10 @@
         <v>1Crowd, Aanshi, Ankur Capital, Beyond Capital, Ennovent, Innospark Ventures, Innovative Directions, Sat Industries, Social Innovation Circle, Sunil Mishra, UBS Optimus Foundation</v>
       </c>
       <c r="G164" t="str">
-        <v>karmahealthcare.in</v>
+        <v>karmahealthcarestaffing.com</v>
+      </c>
+      <c r="H164" t="str">
+        <v>careers@karmahealthcarestaffing.com</v>
       </c>
     </row>
     <row r="165">
@@ -4222,6 +4603,9 @@
       <c r="G166" t="str">
         <v>juicychemistry.com</v>
       </c>
+      <c r="H166" t="str">
+        <v>careers@juicychemistry.com</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -4245,6 +4629,9 @@
       <c r="G167" t="str">
         <v>slyds.com</v>
       </c>
+      <c r="H167" t="str">
+        <v>careers@slyds.com</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -4266,7 +4653,10 @@
         <v>VentureNursery, YourNest Venture Capital</v>
       </c>
       <c r="G168" t="str">
-        <v>arya.ai</v>
+        <v>omnitalk.com</v>
+      </c>
+      <c r="H168" t="str">
+        <v>careers@omnitalk.com</v>
       </c>
     </row>
     <row r="169">
@@ -4337,6 +4727,9 @@
       <c r="G171" t="str">
         <v>numbernagar.com</v>
       </c>
+      <c r="H171" t="str">
+        <v>careers@numbernagar.com</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
@@ -4360,6 +4753,9 @@
       <c r="G172" t="str">
         <v>gxgroup.eu</v>
       </c>
+      <c r="H172" t="str">
+        <v>careers@gxgroup.eu</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
@@ -4383,6 +4779,9 @@
       <c r="G173" t="str">
         <v>hackerrank.com</v>
       </c>
+      <c r="H173" t="str">
+        <v>careers@hackerrank.com</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
@@ -4429,6 +4828,9 @@
       <c r="G175" t="str">
         <v>browntape.com</v>
       </c>
+      <c r="H175" t="str">
+        <v>careers@browntape.com</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
@@ -4452,6 +4854,9 @@
       <c r="G176" t="str">
         <v>zentronlabs.com</v>
       </c>
+      <c r="H176" t="str">
+        <v>careers@zentronlabs.com</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
@@ -4475,6 +4880,9 @@
       <c r="G177" t="str">
         <v>kulzy.com</v>
       </c>
+      <c r="H177" t="str">
+        <v>careers@kulzy.com</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
@@ -4521,6 +4929,9 @@
       <c r="G179" t="str">
         <v>wonobo.com</v>
       </c>
+      <c r="H179" t="str">
+        <v>careers@wonobo.com</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
@@ -4567,6 +4978,9 @@
       <c r="G181" t="str">
         <v>travelkhana.com</v>
       </c>
+      <c r="H181" t="str">
+        <v>careers@travelkhana.com</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
@@ -4613,6 +5027,9 @@
       <c r="G183" t="str">
         <v>nativespecial.com</v>
       </c>
+      <c r="H183" t="str">
+        <v>careers@nativespecial.com</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
@@ -4636,6 +5053,9 @@
       <c r="G184" t="str">
         <v>rmlagtech.com</v>
       </c>
+      <c r="H184" t="str">
+        <v>careers@rmlagtech.com</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
@@ -4657,7 +5077,10 @@
         <v>Deven Lakshmi Chand Bebhia Bebhia, YourNest Venture Capital</v>
       </c>
       <c r="G185" t="str">
-        <v>golflan.com</v>
+        <v>golfland.com</v>
+      </c>
+      <c r="H185" t="str">
+        <v>careers@golfland.com</v>
       </c>
     </row>
     <row r="186">
@@ -4680,7 +5103,10 @@
         <v>Aavishkaar Venture Capital</v>
       </c>
       <c r="G186" t="str">
-        <v>soulfull.co.in</v>
+        <v>soulfullymade.com</v>
+      </c>
+      <c r="H186" t="str">
+        <v>careers@soulfullymade.com</v>
       </c>
     </row>
     <row r="187">
@@ -4703,7 +5129,10 @@
         <v>Aavishkaar Venture Capital, India Quotient, Unilazer Ventures</v>
       </c>
       <c r="G187" t="str">
-        <v>meradoctor.com</v>
+        <v>meradoctorr.com</v>
+      </c>
+      <c r="H187" t="str">
+        <v>careers@meradoctorr.com</v>
       </c>
     </row>
     <row r="188">
@@ -4726,7 +5155,10 @@
         <v>Cadabams Group</v>
       </c>
       <c r="G188" t="str">
-        <v>mindtalk.in</v>
+        <v>mindtalkpsychology.com.au</v>
+      </c>
+      <c r="H188" t="str">
+        <v>careers@mindtalkpsychology.com.au</v>
       </c>
     </row>
     <row r="189">
@@ -4751,6 +5183,9 @@
       <c r="G189" t="str">
         <v>jagaranmf.com</v>
       </c>
+      <c r="H189" t="str">
+        <v>careers@jagaranmf.com</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
@@ -4795,7 +5230,10 @@
         <v>ICICI Venture, Peak XV Partners</v>
       </c>
       <c r="G191" t="str">
-        <v>gocolors.co.in</v>
+        <v>gocolors.com</v>
+      </c>
+      <c r="H191" t="str">
+        <v>careers@gocolors.com</v>
       </c>
     </row>
     <row r="192">
@@ -4820,6 +5258,9 @@
       <c r="G192" t="str">
         <v>paymate.in</v>
       </c>
+      <c r="H192" t="str">
+        <v>careers@paymate.in</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
@@ -4841,7 +5282,10 @@
         <v>Info Edge, SeedFund.in, Sequoia Capital</v>
       </c>
       <c r="G193" t="str">
-        <v>printo.in</v>
+        <v>printograph.com</v>
+      </c>
+      <c r="H193" t="str">
+        <v>careers@printograph.com</v>
       </c>
     </row>
     <row r="194">
@@ -4866,6 +5310,9 @@
       <c r="G194" t="str">
         <v>kredent.com</v>
       </c>
+      <c r="H194" t="str">
+        <v>careers@kredent.com</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
@@ -4889,6 +5336,9 @@
       <c r="G195" t="str">
         <v>games24x7.com</v>
       </c>
+      <c r="H195" t="str">
+        <v>careers@games24x7.com</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
@@ -4912,6 +5362,9 @@
       <c r="G196" t="str">
         <v>yatra.com</v>
       </c>
+      <c r="H196" t="str">
+        <v>careers@yatra.com</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
@@ -4933,7 +5386,10 @@
         <v>Cactus Partners</v>
       </c>
       <c r="G197" t="str">
-        <v/>
+        <v>kapture.ca</v>
+      </c>
+      <c r="H197" t="str">
+        <v>careers@kapture.ca</v>
       </c>
     </row>
     <row r="198">
@@ -4956,7 +5412,10 @@
         <v>Gaja Capital</v>
       </c>
       <c r="G198" t="str">
-        <v/>
+        <v>theindusvalley.in</v>
+      </c>
+      <c r="H198" t="str">
+        <v>careers@theindusvalley.in</v>
       </c>
     </row>
     <row r="199">
@@ -4979,7 +5438,10 @@
         <v>dataAlpha</v>
       </c>
       <c r="G199" t="str">
-        <v/>
+        <v>yolearner.com</v>
+      </c>
+      <c r="H199" t="str">
+        <v>careers@yolearner.com</v>
       </c>
     </row>
     <row r="200">
@@ -5025,7 +5487,10 @@
         <v>Bharat Value Fund</v>
       </c>
       <c r="G201" t="str">
-        <v/>
+        <v>incuspaze.com</v>
+      </c>
+      <c r="H201" t="str">
+        <v>careers@incuspaze.com</v>
       </c>
     </row>
     <row r="202">
@@ -5048,7 +5513,10 @@
         <v>Andrew Parker</v>
       </c>
       <c r="G202" t="str">
-        <v/>
+        <v>mykarehealth.com</v>
+      </c>
+      <c r="H202" t="str">
+        <v>careers@mykarehealth.com</v>
       </c>
     </row>
     <row r="203">
@@ -5071,7 +5539,10 @@
         <v>Yash Raj Films</v>
       </c>
       <c r="G203" t="str">
-        <v/>
+        <v>ruskmedia.com</v>
+      </c>
+      <c r="H203" t="str">
+        <v>careers@ruskmedia.com</v>
       </c>
     </row>
     <row r="204">
@@ -5094,7 +5565,10 @@
         <v>Tilaknagar Industries</v>
       </c>
       <c r="G204" t="str">
-        <v/>
+        <v>bartisans.in</v>
+      </c>
+      <c r="H204" t="str">
+        <v>careers@bartisans.in</v>
       </c>
     </row>
     <row r="205">
@@ -5117,7 +5591,10 @@
         <v>Boundless Ventures</v>
       </c>
       <c r="G205" t="str">
-        <v/>
+        <v>lytmus.io</v>
+      </c>
+      <c r="H205" t="str">
+        <v>careers@lytmus.io</v>
       </c>
     </row>
     <row r="206">
@@ -5140,7 +5617,10 @@
         <v>Ramakant Deshpande</v>
       </c>
       <c r="G206" t="str">
-        <v/>
+        <v>finnovate.in</v>
+      </c>
+      <c r="H206" t="str">
+        <v>careers@finnovate.in</v>
       </c>
     </row>
     <row r="207">
@@ -5186,7 +5666,10 @@
         <v>Stride Ventures</v>
       </c>
       <c r="G208" t="str">
-        <v/>
+        <v>allhomes.com.au</v>
+      </c>
+      <c r="H208" t="str">
+        <v>careers@allhomes.com.au</v>
       </c>
     </row>
     <row r="209">
@@ -5209,7 +5692,10 @@
         <v>Lightspeed Venture Partners</v>
       </c>
       <c r="G209" t="str">
-        <v/>
+        <v>superliving.co.uk</v>
+      </c>
+      <c r="H209" t="str">
+        <v>careers@superliving.co.uk</v>
       </c>
     </row>
     <row r="210">
@@ -5232,7 +5718,10 @@
         <v>JSW Group</v>
       </c>
       <c r="G210" t="str">
-        <v/>
+        <v>project-lithium.com</v>
+      </c>
+      <c r="H210" t="str">
+        <v>careers@project-lithium.com</v>
       </c>
     </row>
     <row r="211">
@@ -5255,7 +5744,10 @@
         <v>Inflection Point Ventures</v>
       </c>
       <c r="G211" t="str">
-        <v/>
+        <v>zavedenia.com</v>
+      </c>
+      <c r="H211" t="str">
+        <v>careers@zavedenia.com</v>
       </c>
     </row>
     <row r="212">
@@ -5278,7 +5770,10 @@
         <v>build3</v>
       </c>
       <c r="G212" t="str">
-        <v/>
+        <v>medi-know.org</v>
+      </c>
+      <c r="H212" t="str">
+        <v>careers@medi-know.org</v>
       </c>
     </row>
     <row r="213">
@@ -5301,7 +5796,10 @@
         <v>Infinity Ventures</v>
       </c>
       <c r="G213" t="str">
-        <v/>
+        <v>saffronstays.com</v>
+      </c>
+      <c r="H213" t="str">
+        <v>careers@saffronstays.com</v>
       </c>
     </row>
     <row r="214">
@@ -5324,7 +5822,10 @@
         <v>Unicorn India Ventures</v>
       </c>
       <c r="G214" t="str">
-        <v/>
+        <v>ikinglobal.com</v>
+      </c>
+      <c r="H214" t="str">
+        <v>careers@ikinglobal.com</v>
       </c>
     </row>
     <row r="215">
@@ -5370,7 +5871,10 @@
         <v>AIFL</v>
       </c>
       <c r="G216" t="str">
-        <v/>
+        <v>roofsol.com</v>
+      </c>
+      <c r="H216" t="str">
+        <v>careers@roofsol.com</v>
       </c>
     </row>
     <row r="217">
@@ -5416,7 +5920,10 @@
         <v>—</v>
       </c>
       <c r="G218" t="str">
-        <v/>
+        <v>squareyards.com</v>
+      </c>
+      <c r="H218" t="str">
+        <v>careers@squareyards.com</v>
       </c>
     </row>
     <row r="219">
@@ -5462,7 +5969,10 @@
         <v>Bhoruka Supply Chain Solutions Holdings</v>
       </c>
       <c r="G220" t="str">
-        <v/>
+        <v>bluetokaicoffee.com</v>
+      </c>
+      <c r="H220" t="str">
+        <v>careers@bluetokaicoffee.com</v>
       </c>
     </row>
     <row r="221">
@@ -5554,7 +6064,10 @@
         <v>Recur Club</v>
       </c>
       <c r="G224" t="str">
-        <v/>
+        <v>unnatisilks.com</v>
+      </c>
+      <c r="H224" t="str">
+        <v>careers@unnatisilks.com</v>
       </c>
     </row>
     <row r="225">
@@ -5600,7 +6113,10 @@
         <v>Meta</v>
       </c>
       <c r="G226" t="str">
-        <v/>
+        <v>creditkarma.com</v>
+      </c>
+      <c r="H226" t="str">
+        <v>careers@creditkarma.com</v>
       </c>
     </row>
     <row r="227">
@@ -5623,7 +6139,10 @@
         <v>Strat Ventures</v>
       </c>
       <c r="G227" t="str">
-        <v/>
+        <v>recykal.com</v>
+      </c>
+      <c r="H227" t="str">
+        <v>careers@recykal.com</v>
       </c>
     </row>
     <row r="228">
@@ -5646,7 +6165,10 @@
         <v>Crizac</v>
       </c>
       <c r="G228" t="str">
-        <v/>
+        <v>foreignadmits.com</v>
+      </c>
+      <c r="H228" t="str">
+        <v>careers@foreignadmits.com</v>
       </c>
     </row>
     <row r="229">
@@ -5692,7 +6214,10 @@
         <v>Rainmatter</v>
       </c>
       <c r="G230" t="str">
-        <v/>
+        <v>karosambhav.com</v>
+      </c>
+      <c r="H230" t="str">
+        <v>careers@karosambhav.com</v>
       </c>
     </row>
     <row r="231">
@@ -5715,7 +6240,10 @@
         <v>Bessemer Venture Partners</v>
       </c>
       <c r="G231" t="str">
-        <v/>
+        <v>vet-i-care.org</v>
+      </c>
+      <c r="H231" t="str">
+        <v>careers@vet-i-care.org</v>
       </c>
     </row>
     <row r="232">
@@ -5784,7 +6312,10 @@
         <v>Indifly Ventures</v>
       </c>
       <c r="G234" t="str">
-        <v/>
+        <v>c-green.se</v>
+      </c>
+      <c r="H234" t="str">
+        <v>careers@c-green.se</v>
       </c>
     </row>
     <row r="235">
@@ -5807,7 +6338,10 @@
         <v>Rainmatter</v>
       </c>
       <c r="G235" t="str">
-        <v/>
+        <v>lissun.app</v>
+      </c>
+      <c r="H235" t="str">
+        <v>careers@lissun.app</v>
       </c>
     </row>
     <row r="236">
@@ -5853,7 +6387,10 @@
         <v>Orbimed</v>
       </c>
       <c r="G237" t="str">
-        <v/>
+        <v>trunativ.co</v>
+      </c>
+      <c r="H237" t="str">
+        <v>careers@trunativ.co</v>
       </c>
     </row>
     <row r="238">
@@ -5899,7 +6436,10 @@
         <v>Atomic Capital</v>
       </c>
       <c r="G239" t="str">
-        <v/>
+        <v>speedio.co.il</v>
+      </c>
+      <c r="H239" t="str">
+        <v>careers@speedio.co.il</v>
       </c>
     </row>
     <row r="240">
@@ -5922,7 +6462,10 @@
         <v>B Capital</v>
       </c>
       <c r="G240" t="str">
-        <v/>
+        <v>solarsquare.in</v>
+      </c>
+      <c r="H240" t="str">
+        <v>careers@solarsquare.in</v>
       </c>
     </row>
     <row r="241">
@@ -5945,7 +6488,10 @@
         <v>Pontaq</v>
       </c>
       <c r="G241" t="str">
-        <v/>
+        <v>trackersuite.com</v>
+      </c>
+      <c r="H241" t="str">
+        <v>careers@trackersuite.com</v>
       </c>
     </row>
     <row r="242">
@@ -5968,7 +6514,10 @@
         <v>Beenext</v>
       </c>
       <c r="G242" t="str">
-        <v/>
+        <v>crestcapital.com</v>
+      </c>
+      <c r="H242" t="str">
+        <v>careers@crestcapital.com</v>
       </c>
     </row>
     <row r="243">
@@ -5991,7 +6540,10 @@
         <v>NSFO</v>
       </c>
       <c r="G243" t="str">
-        <v/>
+        <v>foodstoriesblog.com</v>
+      </c>
+      <c r="H243" t="str">
+        <v>careers@foodstoriesblog.com</v>
       </c>
     </row>
     <row r="244">
@@ -6014,7 +6566,10 @@
         <v>Singularity AMC</v>
       </c>
       <c r="G244" t="str">
-        <v/>
+        <v>autovrse.in</v>
+      </c>
+      <c r="H244" t="str">
+        <v>careers@autovrse.in</v>
       </c>
     </row>
     <row r="245">
@@ -6037,7 +6592,10 @@
         <v>Bessemer Venture Partners</v>
       </c>
       <c r="G245" t="str">
-        <v/>
+        <v>sarvamfx.com</v>
+      </c>
+      <c r="H245" t="str">
+        <v>careers@sarvamfx.com</v>
       </c>
     </row>
     <row r="246">
@@ -6060,7 +6618,10 @@
         <v>Undisclosed</v>
       </c>
       <c r="G246" t="str">
-        <v/>
+        <v>glamour.com</v>
+      </c>
+      <c r="H246" t="str">
+        <v>careers@glamour.com</v>
       </c>
     </row>
     <row r="247">
@@ -6083,7 +6644,10 @@
         <v>Accel</v>
       </c>
       <c r="G247" t="str">
-        <v/>
+        <v>zumutor.com</v>
+      </c>
+      <c r="H247" t="str">
+        <v>careers@zumutor.com</v>
       </c>
     </row>
     <row r="248">
@@ -6106,7 +6670,10 @@
         <v>Accel</v>
       </c>
       <c r="G248" t="str">
-        <v/>
+        <v>rekise.com</v>
+      </c>
+      <c r="H248" t="str">
+        <v>careers@rekise.com</v>
       </c>
     </row>
     <row r="249">
@@ -6129,7 +6696,10 @@
         <v>Info Edge Ventures</v>
       </c>
       <c r="G249" t="str">
-        <v/>
+        <v>lumiqlearn.com</v>
+      </c>
+      <c r="H249" t="str">
+        <v>careers@lumiqlearn.com</v>
       </c>
     </row>
     <row r="250">
@@ -6152,7 +6722,10 @@
         <v>Prosus</v>
       </c>
       <c r="G250" t="str">
-        <v/>
+        <v>lgbtequalitypac.org</v>
+      </c>
+      <c r="H250" t="str">
+        <v>careers@lgbtequalitypac.org</v>
       </c>
     </row>
     <row r="251">
@@ -6198,7 +6771,10 @@
         <v>Rohit Gurunath Sharma</v>
       </c>
       <c r="G252" t="str">
-        <v/>
+        <v>fittr.com</v>
+      </c>
+      <c r="H252" t="str">
+        <v>careers@fittr.com</v>
       </c>
     </row>
     <row r="253">
@@ -6221,7 +6797,10 @@
         <v>247VC</v>
       </c>
       <c r="G253" t="str">
-        <v/>
+        <v>dreamaerospace.in</v>
+      </c>
+      <c r="H253" t="str">
+        <v>careers@dreamaerospace.in</v>
       </c>
     </row>
     <row r="254">
@@ -6244,7 +6823,10 @@
         <v>Ahdritz</v>
       </c>
       <c r="G254" t="str">
-        <v/>
+        <v>madverse.com</v>
+      </c>
+      <c r="H254" t="str">
+        <v>careers@madverse.com</v>
       </c>
     </row>
     <row r="255">
@@ -6267,7 +6849,10 @@
         <v>Unicorn India Ventures</v>
       </c>
       <c r="G255" t="str">
-        <v/>
+        <v>qubehealth.com</v>
+      </c>
+      <c r="H255" t="str">
+        <v>careers@qubehealth.com</v>
       </c>
     </row>
     <row r="256">
@@ -6290,7 +6875,10 @@
         <v>Indian Angel Network</v>
       </c>
       <c r="G256" t="str">
-        <v/>
+        <v>biodimension.in</v>
+      </c>
+      <c r="H256" t="str">
+        <v>careers@biodimension.in</v>
       </c>
     </row>
     <row r="257">
@@ -6313,7 +6901,10 @@
         <v>Inflection Point Ventures</v>
       </c>
       <c r="G257" t="str">
-        <v/>
+        <v>dartlearning.org.au</v>
+      </c>
+      <c r="H257" t="str">
+        <v>careers@dartlearning.org.au</v>
       </c>
     </row>
     <row r="258">
@@ -6336,7 +6927,10 @@
         <v>Earlyseed Ventures</v>
       </c>
       <c r="G258" t="str">
-        <v/>
+        <v>electriq.co.in</v>
+      </c>
+      <c r="H258" t="str">
+        <v>careers@electriq.co.in</v>
       </c>
     </row>
     <row r="259">
@@ -6382,7 +6976,10 @@
         <v>Dharana</v>
       </c>
       <c r="G260" t="str">
-        <v/>
+        <v>mygate.com</v>
+      </c>
+      <c r="H260" t="str">
+        <v>careers@mygate.com</v>
       </c>
     </row>
     <row r="261">
@@ -6474,7 +7071,10 @@
         <v>Peak XV Partners</v>
       </c>
       <c r="G264" t="str">
-        <v/>
+        <v>hoolah.co</v>
+      </c>
+      <c r="H264" t="str">
+        <v>careers@hoolah.co</v>
       </c>
     </row>
     <row r="265">
@@ -6520,7 +7120,10 @@
         <v>Wellingdon Advisors</v>
       </c>
       <c r="G266" t="str">
-        <v/>
+        <v>431theweddingcompany.ca</v>
+      </c>
+      <c r="H266" t="str">
+        <v>careers@431theweddingcompany.ca</v>
       </c>
     </row>
     <row r="267">
@@ -6543,7 +7146,10 @@
         <v>BlackSoil</v>
       </c>
       <c r="G267" t="str">
-        <v/>
+        <v>celebaltech.com</v>
+      </c>
+      <c r="H267" t="str">
+        <v>careers@celebaltech.com</v>
       </c>
     </row>
     <row r="268">
@@ -6589,7 +7195,10 @@
         <v>Enrission India Capital</v>
       </c>
       <c r="G269" t="str">
-        <v/>
+        <v>recurclub.com</v>
+      </c>
+      <c r="H269" t="str">
+        <v>careers@recurclub.com</v>
       </c>
     </row>
     <row r="270">
@@ -6612,7 +7221,10 @@
         <v>Fullerton Carbon Action Fund</v>
       </c>
       <c r="G270" t="str">
-        <v/>
+        <v>hy2gen.com</v>
+      </c>
+      <c r="H270" t="str">
+        <v>careers@hy2gen.com</v>
       </c>
     </row>
     <row r="271">
@@ -6635,7 +7247,10 @@
         <v>Singularity AMC</v>
       </c>
       <c r="G271" t="str">
-        <v/>
+        <v>immuneel.com</v>
+      </c>
+      <c r="H271" t="str">
+        <v>careers@immuneel.com</v>
       </c>
     </row>
     <row r="272">
@@ -6681,7 +7296,10 @@
         <v>Panthera</v>
       </c>
       <c r="G273" t="str">
-        <v/>
+        <v>innefu.com</v>
+      </c>
+      <c r="H273" t="str">
+        <v>careers@innefu.com</v>
       </c>
     </row>
     <row r="274">
@@ -6704,7 +7322,10 @@
         <v>Suraj Nalin</v>
       </c>
       <c r="G274" t="str">
-        <v/>
+        <v>aadyah.com</v>
+      </c>
+      <c r="H274" t="str">
+        <v>careers@aadyah.com</v>
       </c>
     </row>
     <row r="275">
@@ -6727,7 +7348,10 @@
         <v>Genrobotics</v>
       </c>
       <c r="G275" t="str">
-        <v/>
+        <v>estrotech.in</v>
+      </c>
+      <c r="H275" t="str">
+        <v>careers@estrotech.in</v>
       </c>
     </row>
     <row r="276">
@@ -6750,7 +7374,10 @@
         <v>Ekta Kapoor Ravi</v>
       </c>
       <c r="G276" t="str">
-        <v/>
+        <v>ekatraiot.com</v>
+      </c>
+      <c r="H276" t="str">
+        <v>careers@ekatraiot.com</v>
       </c>
     </row>
     <row r="277">
@@ -6773,7 +7400,10 @@
         <v>Bakkt</v>
       </c>
       <c r="G277" t="str">
-        <v/>
+        <v>transchem.net</v>
+      </c>
+      <c r="H277" t="str">
+        <v>careers@transchem.net</v>
       </c>
     </row>
     <row r="278">
@@ -6796,7 +7426,10 @@
         <v>Peak XV Partners</v>
       </c>
       <c r="G278" t="str">
-        <v/>
+        <v>first20.club</v>
+      </c>
+      <c r="H278" t="str">
+        <v>careers@first20.club</v>
       </c>
     </row>
     <row r="279">
@@ -6842,7 +7475,10 @@
         <v>Sony Innovation Fund</v>
       </c>
       <c r="G280" t="str">
-        <v/>
+        <v>werize.com</v>
+      </c>
+      <c r="H280" t="str">
+        <v>careers@werize.com</v>
       </c>
     </row>
     <row r="281">
@@ -6911,7 +7547,10 @@
         <v>PixelSky Capital</v>
       </c>
       <c r="G283" t="str">
-        <v/>
+        <v>greenpowersystems.co.in</v>
+      </c>
+      <c r="H283" t="str">
+        <v>careers@greenpowersystems.co.in</v>
       </c>
     </row>
     <row r="284">
@@ -6934,7 +7573,10 @@
         <v>Athera</v>
       </c>
       <c r="G284" t="str">
-        <v/>
+        <v>propsoch.com</v>
+      </c>
+      <c r="H284" t="str">
+        <v>careers@propsoch.com</v>
       </c>
     </row>
     <row r="285">
@@ -6957,7 +7599,10 @@
         <v>OTP Ventures</v>
       </c>
       <c r="G285" t="str">
-        <v/>
+        <v>phaboard.org</v>
+      </c>
+      <c r="H285" t="str">
+        <v>careers@phaboard.org</v>
       </c>
     </row>
     <row r="286">
@@ -6980,7 +7625,10 @@
         <v>V3 Ventures</v>
       </c>
       <c r="G286" t="str">
-        <v/>
+        <v>fraganote.com</v>
+      </c>
+      <c r="H286" t="str">
+        <v>careers@fraganote.com</v>
       </c>
     </row>
     <row r="287">
@@ -7003,7 +7651,10 @@
         <v>Shilpa Shetty Kundra</v>
       </c>
       <c r="G287" t="str">
-        <v/>
+        <v>rosaanddaniel.com</v>
+      </c>
+      <c r="H287" t="str">
+        <v>careers@rosaanddaniel.com</v>
       </c>
     </row>
     <row r="288">
@@ -7026,7 +7677,10 @@
         <v>Beenext</v>
       </c>
       <c r="G288" t="str">
-        <v/>
+        <v>prolearners.lk</v>
+      </c>
+      <c r="H288" t="str">
+        <v>careers@prolearners.lk</v>
       </c>
     </row>
     <row r="289">
@@ -7095,7 +7749,10 @@
         <v>Antler</v>
       </c>
       <c r="G291" t="str">
-        <v/>
+        <v>rovia.com</v>
+      </c>
+      <c r="H291" t="str">
+        <v>careers@rovia.com</v>
       </c>
     </row>
     <row r="292">
@@ -7118,7 +7775,10 @@
         <v>Capitar Ventures</v>
       </c>
       <c r="G292" t="str">
-        <v/>
+        <v>simplenergy.us</v>
+      </c>
+      <c r="H292" t="str">
+        <v>careers@simplenergy.us</v>
       </c>
     </row>
     <row r="293">
@@ -7164,7 +7824,10 @@
         <v>Lotus Herbals</v>
       </c>
       <c r="G294" t="str">
-        <v/>
+        <v>korinmills.com</v>
+      </c>
+      <c r="H294" t="str">
+        <v>careers@korinmills.com</v>
       </c>
     </row>
     <row r="295">
@@ -7187,7 +7850,10 @@
         <v>Anushka Sharma</v>
       </c>
       <c r="G295" t="str">
-        <v/>
+        <v>agilitas.be</v>
+      </c>
+      <c r="H295" t="str">
+        <v>careers@agilitas.be</v>
       </c>
     </row>
     <row r="296">
@@ -7210,7 +7876,10 @@
         <v>Vertex Ventures</v>
       </c>
       <c r="G296" t="str">
-        <v/>
+        <v>anveshan.farm</v>
+      </c>
+      <c r="H296" t="str">
+        <v>careers@anveshan.farm</v>
       </c>
     </row>
     <row r="297">
@@ -7233,7 +7902,10 @@
         <v>AIFL</v>
       </c>
       <c r="G297" t="str">
-        <v/>
+        <v>myevolvegroup.com</v>
+      </c>
+      <c r="H297" t="str">
+        <v>careers@myevolvegroup.com</v>
       </c>
     </row>
     <row r="298">
@@ -7279,7 +7951,10 @@
         <v>IvyCap Ventures</v>
       </c>
       <c r="G299" t="str">
-        <v/>
+        <v>tiealign.com</v>
+      </c>
+      <c r="H299" t="str">
+        <v>careers@tiealign.com</v>
       </c>
     </row>
     <row r="300">
@@ -7348,7 +8023,10 @@
         <v>Arvind Choudhary</v>
       </c>
       <c r="G302" t="str">
-        <v/>
+        <v>bucketlisttoursbybarb.com</v>
+      </c>
+      <c r="H302" t="str">
+        <v>careers@bucketlisttoursbybarb.com</v>
       </c>
     </row>
     <row r="303">
@@ -7371,7 +8049,10 @@
         <v>Bertelsmann India Investments</v>
       </c>
       <c r="G303" t="str">
-        <v/>
+        <v>fairdealmarketing.com</v>
+      </c>
+      <c r="H303" t="str">
+        <v>careers@fairdealmarketing.com</v>
       </c>
     </row>
     <row r="304">
@@ -7394,7 +8075,10 @@
         <v>GII</v>
       </c>
       <c r="G304" t="str">
-        <v/>
+        <v>yohohongkong.com</v>
+      </c>
+      <c r="H304" t="str">
+        <v>careers@yohohongkong.com</v>
       </c>
     </row>
     <row r="305">
@@ -7463,7 +8147,10 @@
         <v>Kriti Sanon</v>
       </c>
       <c r="G307" t="str">
-        <v/>
+        <v>giva.co</v>
+      </c>
+      <c r="H307" t="str">
+        <v>careers@giva.co</v>
       </c>
     </row>
     <row r="308">
@@ -7486,7 +8173,10 @@
         <v>Info Edge</v>
       </c>
       <c r="G308" t="str">
-        <v/>
+        <v>yesmadam.com</v>
+      </c>
+      <c r="H308" t="str">
+        <v>careers@yesmadam.com</v>
       </c>
     </row>
     <row r="309">
@@ -7509,7 +8199,10 @@
         <v>Hero Enterprise Partner Ventures</v>
       </c>
       <c r="G309" t="str">
-        <v/>
+        <v>abcoffee.in</v>
+      </c>
+      <c r="H309" t="str">
+        <v>careers@abcoffee.in</v>
       </c>
     </row>
     <row r="310">
@@ -7532,7 +8225,10 @@
         <v>Deepak Gupta</v>
       </c>
       <c r="G310" t="str">
-        <v/>
+        <v>gabit.eu</v>
+      </c>
+      <c r="H310" t="str">
+        <v>careers@gabit.eu</v>
       </c>
     </row>
     <row r="311">
@@ -7555,7 +8251,10 @@
         <v>Sthira Partners</v>
       </c>
       <c r="G311" t="str">
-        <v/>
+        <v>tistmedia.in</v>
+      </c>
+      <c r="H311" t="str">
+        <v>careers@tistmedia.in</v>
       </c>
     </row>
     <row r="312">
@@ -7578,7 +8277,10 @@
         <v>-</v>
       </c>
       <c r="G312" t="str">
-        <v/>
+        <v>solfin.com.ve</v>
+      </c>
+      <c r="H312" t="str">
+        <v>careers@solfin.com.ve</v>
       </c>
     </row>
     <row r="313">
@@ -7601,7 +8303,10 @@
         <v>Big Bets</v>
       </c>
       <c r="G313" t="str">
-        <v/>
+        <v>metafy.gg</v>
+      </c>
+      <c r="H313" t="str">
+        <v>careers@metafy.gg</v>
       </c>
     </row>
     <row r="314">
@@ -7624,7 +8329,10 @@
         <v>Adani Power</v>
       </c>
       <c r="G314" t="str">
-        <v/>
+        <v>jppowerventures.com</v>
+      </c>
+      <c r="H314" t="str">
+        <v>careers@jppowerventures.com</v>
       </c>
     </row>
     <row r="315">
@@ -7647,7 +8355,10 @@
         <v>InCred Capital</v>
       </c>
       <c r="G315" t="str">
-        <v/>
+        <v>vemtechnologies.com</v>
+      </c>
+      <c r="H315" t="str">
+        <v>careers@vemtechnologies.com</v>
       </c>
     </row>
     <row r="316">
@@ -7670,7 +8381,10 @@
         <v>Blume Founders Fund</v>
       </c>
       <c r="G316" t="str">
-        <v/>
+        <v>mythiki.gr</v>
+      </c>
+      <c r="H316" t="str">
+        <v>careers@mythiki.gr</v>
       </c>
     </row>
     <row r="317">
@@ -7693,7 +8407,10 @@
         <v>General Catalyst</v>
       </c>
       <c r="G317" t="str">
-        <v/>
+        <v>scapia.cards</v>
+      </c>
+      <c r="H317" t="str">
+        <v>careers@scapia.cards</v>
       </c>
     </row>
     <row r="318">
@@ -7739,7 +8456,10 @@
         <v>Indian Angel Network</v>
       </c>
       <c r="G319" t="str">
-        <v/>
+        <v>anscer.com</v>
+      </c>
+      <c r="H319" t="str">
+        <v>careers@anscer.com</v>
       </c>
     </row>
     <row r="320">
@@ -7762,7 +8482,10 @@
         <v>Temasek</v>
       </c>
       <c r="G320" t="str">
-        <v/>
+        <v>upgrade.com</v>
+      </c>
+      <c r="H320" t="str">
+        <v>careers@upgrade.com</v>
       </c>
     </row>
     <row r="321">
@@ -7808,7 +8531,10 @@
         <v>Aeravti Ventures</v>
       </c>
       <c r="G322" t="str">
-        <v/>
+        <v>onofrio.com</v>
+      </c>
+      <c r="H322" t="str">
+        <v>careers@onofrio.com</v>
       </c>
     </row>
     <row r="323">
@@ -7831,7 +8557,10 @@
         <v>Hindustan Times</v>
       </c>
       <c r="G323" t="str">
-        <v/>
+        <v>damrooplus.com</v>
+      </c>
+      <c r="H323" t="str">
+        <v>careers@damrooplus.com</v>
       </c>
     </row>
     <row r="324">
@@ -7854,7 +8583,10 @@
         <v>Government of Canada</v>
       </c>
       <c r="G324" t="str">
-        <v/>
+        <v>ntwist.com</v>
+      </c>
+      <c r="H324" t="str">
+        <v>careers@ntwist.com</v>
       </c>
     </row>
     <row r="325">
@@ -7877,7 +8609,10 @@
         <v>Alteria Capital</v>
       </c>
       <c r="G325" t="str">
-        <v/>
+        <v>countrydelight.in</v>
+      </c>
+      <c r="H325" t="str">
+        <v>careers@countrydelight.in</v>
       </c>
     </row>
     <row r="326">
@@ -7900,7 +8635,10 @@
         <v>Rainmatter</v>
       </c>
       <c r="G326" t="str">
-        <v/>
+        <v>kalfcu.or.kr</v>
+      </c>
+      <c r="H326" t="str">
+        <v>careers@kalfcu.or.kr</v>
       </c>
     </row>
     <row r="327">
@@ -7923,7 +8661,10 @@
         <v>Advent International</v>
       </c>
       <c r="G327" t="str">
-        <v/>
+        <v>isconbalajifoods.com</v>
+      </c>
+      <c r="H327" t="str">
+        <v>careers@isconbalajifoods.com</v>
       </c>
     </row>
     <row r="328">
@@ -7946,7 +8687,10 @@
         <v>HDFC Bank</v>
       </c>
       <c r="G328" t="str">
-        <v/>
+        <v>dhiway.com</v>
+      </c>
+      <c r="H328" t="str">
+        <v>careers@dhiway.com</v>
       </c>
     </row>
     <row r="329">
@@ -8015,7 +8759,10 @@
         <v>VideoCX</v>
       </c>
       <c r="G331" t="str">
-        <v/>
+        <v>finsprings.net</v>
+      </c>
+      <c r="H331" t="str">
+        <v>careers@finsprings.net</v>
       </c>
     </row>
     <row r="332">
@@ -8038,7 +8785,10 @@
         <v>HDFC Bank</v>
       </c>
       <c r="G332" t="str">
-        <v/>
+        <v>valuenable.in</v>
+      </c>
+      <c r="H332" t="str">
+        <v>careers@valuenable.in</v>
       </c>
     </row>
     <row r="333">
@@ -8061,7 +8811,10 @@
         <v>HDFC Bank</v>
       </c>
       <c r="G333" t="str">
-        <v/>
+        <v>proplegit.com</v>
+      </c>
+      <c r="H333" t="str">
+        <v>careers@proplegit.com</v>
       </c>
     </row>
     <row r="334">
@@ -8084,7 +8837,10 @@
         <v>HDFC Bank</v>
       </c>
       <c r="G334" t="str">
-        <v/>
+        <v>finsall.com</v>
+      </c>
+      <c r="H334" t="str">
+        <v>careers@finsall.com</v>
       </c>
     </row>
     <row r="335">
@@ -8176,7 +8932,10 @@
         <v>HDFC Bank</v>
       </c>
       <c r="G338" t="str">
-        <v/>
+        <v>entitledto.co.uk</v>
+      </c>
+      <c r="H338" t="str">
+        <v>careers@entitledto.co.uk</v>
       </c>
     </row>
     <row r="339">
@@ -8199,7 +8958,10 @@
         <v>Prosus</v>
       </c>
       <c r="G339" t="str">
-        <v/>
+        <v>rapidotrains.com</v>
+      </c>
+      <c r="H339" t="str">
+        <v>careers@rapidotrains.com</v>
       </c>
     </row>
     <row r="340">
@@ -8222,7 +8984,10 @@
         <v>Anrf</v>
       </c>
       <c r="G340" t="str">
-        <v/>
+        <v>dhruvaspace.com</v>
+      </c>
+      <c r="H340" t="str">
+        <v>careers@dhruvaspace.com</v>
       </c>
     </row>
     <row r="341">
@@ -8245,7 +9010,10 @@
         <v>-</v>
       </c>
       <c r="G341" t="str">
-        <v/>
+        <v>cra-online.org</v>
+      </c>
+      <c r="H341" t="str">
+        <v>careers@cra-online.org</v>
       </c>
     </row>
     <row r="342">
@@ -8337,7 +9105,10 @@
         <v>Zoho</v>
       </c>
       <c r="G345" t="str">
-        <v/>
+        <v>ondc.org</v>
+      </c>
+      <c r="H345" t="str">
+        <v>careers@ondc.org</v>
       </c>
     </row>
     <row r="346">
@@ -8360,7 +9131,10 @@
         <v>Titan Capital</v>
       </c>
       <c r="G346" t="str">
-        <v/>
+        <v>instafix.com</v>
+      </c>
+      <c r="H346" t="str">
+        <v>careers@instafix.com</v>
       </c>
     </row>
     <row r="347">
@@ -8452,7 +9226,10 @@
         <v>Triton Investment Advisors</v>
       </c>
       <c r="G350" t="str">
-        <v/>
+        <v>scikiq.com</v>
+      </c>
+      <c r="H350" t="str">
+        <v>careers@scikiq.com</v>
       </c>
     </row>
     <row r="351">
@@ -8475,7 +9252,10 @@
         <v>V3 Ventures</v>
       </c>
       <c r="G351" t="str">
-        <v/>
+        <v>dilfoods.in</v>
+      </c>
+      <c r="H351" t="str">
+        <v>careers@dilfoods.in</v>
       </c>
     </row>
     <row r="352">
@@ -8498,7 +9278,10 @@
         <v>Abler Nordic, Carpediem Capital</v>
       </c>
       <c r="G352" t="str">
-        <v/>
+        <v>sindhujamicrocredit.com</v>
+      </c>
+      <c r="H352" t="str">
+        <v>careers@sindhujamicrocredit.com</v>
       </c>
     </row>
     <row r="353">
@@ -8659,7 +9442,10 @@
         <v>Indian Angel Network, Vertex Ventures</v>
       </c>
       <c r="G359" t="str">
-        <v/>
+        <v>bigendiandata.com</v>
+      </c>
+      <c r="H359" t="str">
+        <v>careers@bigendiandata.com</v>
       </c>
     </row>
     <row r="360">
@@ -8682,7 +9468,10 @@
         <v>Mirova, FMO</v>
       </c>
       <c r="G360" t="str">
-        <v/>
+        <v>ecofy.net.au</v>
+      </c>
+      <c r="H360" t="str">
+        <v>careers@ecofy.net.au</v>
       </c>
     </row>
     <row r="361">
@@ -8728,7 +9517,10 @@
         <v>Physics Wallah</v>
       </c>
       <c r="G362" t="str">
-        <v/>
+        <v>sarrthiias.com</v>
+      </c>
+      <c r="H362" t="str">
+        <v>careers@sarrthiias.com</v>
       </c>
     </row>
     <row r="363">
@@ -8797,7 +9589,10 @@
         <v>-</v>
       </c>
       <c r="G365" t="str">
-        <v/>
+        <v>pinsecor.es</v>
+      </c>
+      <c r="H365" t="str">
+        <v>careers@pinsecor.es</v>
       </c>
     </row>
     <row r="366">
@@ -8820,7 +9615,10 @@
         <v>Lachy Groom, Bain Capital Ventures</v>
       </c>
       <c r="G366" t="str">
-        <v/>
+        <v>pronto.io</v>
+      </c>
+      <c r="H366" t="str">
+        <v>careers@pronto.io</v>
       </c>
     </row>
     <row r="367">
@@ -8843,7 +9641,10 @@
         <v>ManchesterStory Group</v>
       </c>
       <c r="G367" t="str">
-        <v/>
+        <v>xcalibercontainer.com</v>
+      </c>
+      <c r="H367" t="str">
+        <v>careers@xcalibercontainer.com</v>
       </c>
     </row>
     <row r="368">
@@ -8866,7 +9667,10 @@
         <v>Prospect Capital Management</v>
       </c>
       <c r="G368" t="str">
-        <v/>
+        <v>securityfiresystems.com</v>
+      </c>
+      <c r="H368" t="str">
+        <v>careers@securityfiresystems.com</v>
       </c>
     </row>
     <row r="369">
@@ -8912,7 +9716,10 @@
         <v>Piper Serica</v>
       </c>
       <c r="G370" t="str">
-        <v/>
+        <v>vobiz.fr</v>
+      </c>
+      <c r="H370" t="str">
+        <v>careers@vobiz.fr</v>
       </c>
     </row>
     <row r="371">
@@ -8981,7 +9788,10 @@
         <v>Atomic Capital</v>
       </c>
       <c r="G373" t="str">
-        <v/>
+        <v>healthfab.in</v>
+      </c>
+      <c r="H373" t="str">
+        <v>careers@healthfab.in</v>
       </c>
     </row>
     <row r="374">
@@ -9004,7 +9814,10 @@
         <v>Fireside Ventures</v>
       </c>
       <c r="G374" t="str">
-        <v/>
+        <v>kisahdunia.com</v>
+      </c>
+      <c r="H374" t="str">
+        <v>careers@kisahdunia.com</v>
       </c>
     </row>
     <row r="375">
@@ -9027,7 +9840,10 @@
         <v>Fireside Ventures</v>
       </c>
       <c r="G375" t="str">
-        <v/>
+        <v>chosenpeople.com</v>
+      </c>
+      <c r="H375" t="str">
+        <v>careers@chosenpeople.com</v>
       </c>
     </row>
     <row r="376">
@@ -9050,7 +9866,10 @@
         <v>Earthfund</v>
       </c>
       <c r="G376" t="str">
-        <v/>
+        <v>aurma.ru</v>
+      </c>
+      <c r="H376" t="str">
+        <v>careers@aurma.ru</v>
       </c>
     </row>
     <row r="377">
@@ -9096,7 +9915,10 @@
         <v>Rainmatter</v>
       </c>
       <c r="G378" t="str">
-        <v/>
+        <v>novorbis.com.br</v>
+      </c>
+      <c r="H378" t="str">
+        <v>careers@novorbis.com.br</v>
       </c>
     </row>
     <row r="379">
@@ -9142,7 +9964,10 @@
         <v>Bharat Forge</v>
       </c>
       <c r="G380" t="str">
-        <v/>
+        <v>fortunauae.com</v>
+      </c>
+      <c r="H380" t="str">
+        <v>careers@fortunauae.com</v>
       </c>
     </row>
     <row r="381">
@@ -9165,7 +9990,10 @@
         <v>Inflection Point Ventures</v>
       </c>
       <c r="G381" t="str">
-        <v/>
+        <v>ctruh.com</v>
+      </c>
+      <c r="H381" t="str">
+        <v>careers@ctruh.com</v>
       </c>
     </row>
     <row r="382">
@@ -9188,7 +10016,10 @@
         <v>GEF Capital Partners</v>
       </c>
       <c r="G382" t="str">
-        <v/>
+        <v>kimballmidwest.com</v>
+      </c>
+      <c r="H382" t="str">
+        <v>careers@kimballmidwest.com</v>
       </c>
     </row>
     <row r="383">
@@ -9211,7 +10042,10 @@
         <v>Futura Surgicare</v>
       </c>
       <c r="G383" t="str">
-        <v/>
+        <v>rivarpmedical.com</v>
+      </c>
+      <c r="H383" t="str">
+        <v>careers@rivarpmedical.com</v>
       </c>
     </row>
     <row r="384">
@@ -9234,7 +10068,10 @@
         <v>Finvolve</v>
       </c>
       <c r="G384" t="str">
-        <v/>
+        <v>vikraoceantech.com</v>
+      </c>
+      <c r="H384" t="str">
+        <v>careers@vikraoceantech.com</v>
       </c>
     </row>
     <row r="385">
@@ -9257,7 +10094,10 @@
         <v>Subhkam Ventures</v>
       </c>
       <c r="G385" t="str">
-        <v/>
+        <v>sprect.com</v>
+      </c>
+      <c r="H385" t="str">
+        <v>careers@sprect.com</v>
       </c>
     </row>
     <row r="386">
@@ -9280,7 +10120,10 @@
         <v>Indian Angel Network</v>
       </c>
       <c r="G386" t="str">
-        <v/>
+        <v>sportvot.com</v>
+      </c>
+      <c r="H386" t="str">
+        <v>careers@sportvot.com</v>
       </c>
     </row>
     <row r="387">
@@ -9303,7 +10146,10 @@
         <v>State Bank of India</v>
       </c>
       <c r="G387" t="str">
-        <v/>
+        <v>sahamati.org.in</v>
+      </c>
+      <c r="H387" t="str">
+        <v>careers@sahamati.org.in</v>
       </c>
     </row>
     <row r="388">
@@ -9326,7 +10172,10 @@
         <v>Accel</v>
       </c>
       <c r="G388" t="str">
-        <v/>
+        <v>sahibinden.com</v>
+      </c>
+      <c r="H388" t="str">
+        <v>careers@sahibinden.com</v>
       </c>
     </row>
     <row r="389">
@@ -9372,7 +10221,10 @@
         <v>Transition VC</v>
       </c>
       <c r="G390" t="str">
-        <v/>
+        <v>prithu.in</v>
+      </c>
+      <c r="H390" t="str">
+        <v>careers@prithu.in</v>
       </c>
     </row>
     <row r="391">
@@ -9395,7 +10247,10 @@
         <v>Cap Alpha</v>
       </c>
       <c r="G391" t="str">
-        <v/>
+        <v>houseofchikankari.in</v>
+      </c>
+      <c r="H391" t="str">
+        <v>careers@houseofchikankari.in</v>
       </c>
     </row>
     <row r="392">
@@ -9418,7 +10273,10 @@
         <v>TDV Partners</v>
       </c>
       <c r="G392" t="str">
-        <v/>
+        <v>kovona.cz</v>
+      </c>
+      <c r="H392" t="str">
+        <v>careers@kovona.cz</v>
       </c>
     </row>
     <row r="393">
@@ -9441,7 +10299,10 @@
         <v>SIG Venture Capital</v>
       </c>
       <c r="G393" t="str">
-        <v/>
+        <v>snabb-it.cl</v>
+      </c>
+      <c r="H393" t="str">
+        <v>careers@snabb-it.cl</v>
       </c>
     </row>
     <row r="394">
@@ -9464,7 +10325,10 @@
         <v>Mirova</v>
       </c>
       <c r="G394" t="str">
-        <v/>
+        <v>batterysmart.in</v>
+      </c>
+      <c r="H394" t="str">
+        <v>careers@batterysmart.in</v>
       </c>
     </row>
     <row r="395">
@@ -9487,7 +10351,10 @@
         <v>Grand View Research</v>
       </c>
       <c r="G395" t="str">
-        <v/>
+        <v>3dviewer.net</v>
+      </c>
+      <c r="H395" t="str">
+        <v>careers@3dviewer.net</v>
       </c>
     </row>
     <row r="396">
@@ -9510,7 +10377,10 @@
         <v>IvyCap Ventures</v>
       </c>
       <c r="G396" t="str">
-        <v/>
+        <v>hyugalife.com</v>
+      </c>
+      <c r="H396" t="str">
+        <v>careers@hyugalife.com</v>
       </c>
     </row>
     <row r="397">
@@ -9533,7 +10403,10 @@
         <v>Dallas Venture Capital</v>
       </c>
       <c r="G397" t="str">
-        <v/>
+        <v>mojrowerowy.com</v>
+      </c>
+      <c r="H397" t="str">
+        <v>careers@mojrowerowy.com</v>
       </c>
     </row>
     <row r="398">
@@ -9556,7 +10429,10 @@
         <v>Innoven Capital</v>
       </c>
       <c r="G398" t="str">
-        <v/>
+        <v>novio-media.jp</v>
+      </c>
+      <c r="H398" t="str">
+        <v>careers@novio-media.jp</v>
       </c>
     </row>
     <row r="399">
@@ -9602,7 +10478,10 @@
         <v>Swishin Ventures</v>
       </c>
       <c r="G400" t="str">
-        <v/>
+        <v>localtreefellers.com</v>
+      </c>
+      <c r="H400" t="str">
+        <v>careers@localtreefellers.com</v>
       </c>
     </row>
     <row r="401">
@@ -9625,7 +10504,10 @@
         <v>Accel</v>
       </c>
       <c r="G401" t="str">
-        <v/>
+        <v>oolkay.com</v>
+      </c>
+      <c r="H401" t="str">
+        <v>careers@oolkay.com</v>
       </c>
     </row>
     <row r="402">
@@ -9671,7 +10553,10 @@
         <v>Namita Thapar</v>
       </c>
       <c r="G403" t="str">
-        <v/>
+        <v>artociti.com</v>
+      </c>
+      <c r="H403" t="str">
+        <v>careers@artociti.com</v>
       </c>
     </row>
     <row r="404">
@@ -9694,7 +10579,10 @@
         <v>Unicorn India Ventures</v>
       </c>
       <c r="G404" t="str">
-        <v/>
+        <v>deepalgorithms.in</v>
+      </c>
+      <c r="H404" t="str">
+        <v>careers@deepalgorithms.in</v>
       </c>
     </row>
     <row r="405">
@@ -9740,7 +10628,10 @@
         <v>Vineeta Singh</v>
       </c>
       <c r="G406" t="str">
-        <v/>
+        <v>soilsense.io</v>
+      </c>
+      <c r="H406" t="str">
+        <v>careers@soilsense.io</v>
       </c>
     </row>
     <row r="407">
@@ -9763,7 +10654,10 @@
         <v>Omnivore</v>
       </c>
       <c r="G407" t="str">
-        <v/>
+        <v>stcharleshealthcare.org</v>
+      </c>
+      <c r="H407" t="str">
+        <v>careers@stcharleshealthcare.org</v>
       </c>
     </row>
     <row r="408">
@@ -9786,7 +10680,10 @@
         <v>Ritesh Agarwal</v>
       </c>
       <c r="G408" t="str">
-        <v/>
+        <v>awsumnews.co.za</v>
+      </c>
+      <c r="H408" t="str">
+        <v>careers@awsumnews.co.za</v>
       </c>
     </row>
     <row r="409">
@@ -9832,7 +10729,10 @@
         <v>ICMG Group</v>
       </c>
       <c r="G410" t="str">
-        <v/>
+        <v>grest.in</v>
+      </c>
+      <c r="H410" t="str">
+        <v>careers@grest.in</v>
       </c>
     </row>
     <row r="411">
@@ -9855,7 +10755,10 @@
         <v>LC Nueva AIF</v>
       </c>
       <c r="G411" t="str">
-        <v/>
+        <v>alayam.com</v>
+      </c>
+      <c r="H411" t="str">
+        <v>careers@alayam.com</v>
       </c>
     </row>
     <row r="412">
@@ -9924,7 +10827,10 @@
         <v>ICICI Venture</v>
       </c>
       <c r="G414" t="str">
-        <v/>
+        <v>agrowallied.in</v>
+      </c>
+      <c r="H414" t="str">
+        <v>careers@agrowallied.in</v>
       </c>
     </row>
     <row r="415">
@@ -9947,7 +10853,10 @@
         <v>Ajinkya Rahane</v>
       </c>
       <c r="G415" t="str">
-        <v/>
+        <v>chupps.com</v>
+      </c>
+      <c r="H415" t="str">
+        <v>careers@chupps.com</v>
       </c>
     </row>
     <row r="416">
@@ -9993,7 +10902,10 @@
         <v>AWE Funds</v>
       </c>
       <c r="G417" t="str">
-        <v/>
+        <v>digitalpaani.com</v>
+      </c>
+      <c r="H417" t="str">
+        <v>careers@digitalpaani.com</v>
       </c>
     </row>
     <row r="418">
@@ -10062,7 +10974,10 @@
         <v>Rainmatter</v>
       </c>
       <c r="G420" t="str">
-        <v/>
+        <v>lawyered.in</v>
+      </c>
+      <c r="H420" t="str">
+        <v>careers@lawyered.in</v>
       </c>
     </row>
     <row r="421">
@@ -10108,7 +11023,10 @@
         <v>SucSEED Indovation</v>
       </c>
       <c r="G422" t="str">
-        <v/>
+        <v>truscholar.io</v>
+      </c>
+      <c r="H422" t="str">
+        <v>careers@truscholar.io</v>
       </c>
     </row>
     <row r="423">
@@ -10131,7 +11049,10 @@
         <v>Sauce</v>
       </c>
       <c r="G423" t="str">
-        <v/>
+        <v>hoccokhi.vn</v>
+      </c>
+      <c r="H423" t="str">
+        <v>careers@hoccokhi.vn</v>
       </c>
     </row>
     <row r="424">
@@ -10154,7 +11075,10 @@
         <v>Zee Entertainment Enterprises</v>
       </c>
       <c r="G424" t="str">
-        <v/>
+        <v>phantom-fx.com</v>
+      </c>
+      <c r="H424" t="str">
+        <v>careers@phantom-fx.com</v>
       </c>
     </row>
     <row r="425">
@@ -10177,7 +11101,10 @@
         <v>Promaft Partners</v>
       </c>
       <c r="G425" t="str">
-        <v/>
+        <v>thehosteller.com</v>
+      </c>
+      <c r="H425" t="str">
+        <v>careers@thehosteller.com</v>
       </c>
     </row>
     <row r="426">
@@ -10200,7 +11127,10 @@
         <v>BIG Global Investments JSC</v>
       </c>
       <c r="G426" t="str">
-        <v/>
+        <v>xdcam-user.com</v>
+      </c>
+      <c r="H426" t="str">
+        <v>careers@xdcam-user.com</v>
       </c>
     </row>
     <row r="427">
@@ -10223,7 +11153,10 @@
         <v>Chemelex</v>
       </c>
       <c r="G427" t="str">
-        <v/>
+        <v>algolia.com</v>
+      </c>
+      <c r="H427" t="str">
+        <v>careers@algolia.com</v>
       </c>
     </row>
     <row r="428">
@@ -10246,7 +11179,10 @@
         <v>Pentathlon Ventures</v>
       </c>
       <c r="G428" t="str">
-        <v/>
+        <v>intellithink.in</v>
+      </c>
+      <c r="H428" t="str">
+        <v>careers@intellithink.in</v>
       </c>
     </row>
     <row r="429">
@@ -10269,7 +11205,10 @@
         <v>British International Investment</v>
       </c>
       <c r="G429" t="str">
-        <v/>
+        <v>polaris.com</v>
+      </c>
+      <c r="H429" t="str">
+        <v>careers@polaris.com</v>
       </c>
     </row>
     <row r="430">
@@ -10292,7 +11231,10 @@
         <v>Inflection Point Ventures</v>
       </c>
       <c r="G430" t="str">
-        <v/>
+        <v>cohomacoffee.com</v>
+      </c>
+      <c r="H430" t="str">
+        <v>careers@cohomacoffee.com</v>
       </c>
     </row>
     <row r="431">
@@ -10338,7 +11280,10 @@
         <v>Albinder Dhindsa</v>
       </c>
       <c r="G432" t="str">
-        <v/>
+        <v>helium10.com</v>
+      </c>
+      <c r="H432" t="str">
+        <v>careers@helium10.com</v>
       </c>
     </row>
     <row r="433">
@@ -10361,7 +11306,10 @@
         <v>Draper</v>
       </c>
       <c r="G433" t="str">
-        <v/>
+        <v>ivory.co.il</v>
+      </c>
+      <c r="H433" t="str">
+        <v>careers@ivory.co.il</v>
       </c>
     </row>
     <row r="434">
@@ -10384,7 +11332,10 @@
         <v>SIG Venture Capital</v>
       </c>
       <c r="G434" t="str">
-        <v/>
+        <v>gobblecube.ai</v>
+      </c>
+      <c r="H434" t="str">
+        <v>careers@gobblecube.ai</v>
       </c>
     </row>
     <row r="435">
@@ -10407,7 +11358,10 @@
         <v>Volrado Venture Partners</v>
       </c>
       <c r="G435" t="str">
-        <v/>
+        <v>healync.com</v>
+      </c>
+      <c r="H435" t="str">
+        <v>careers@healync.com</v>
       </c>
     </row>
     <row r="436">
@@ -10430,7 +11384,10 @@
         <v>Everstone Capital</v>
       </c>
       <c r="G436" t="str">
-        <v/>
+        <v>apotheconpharma.com</v>
+      </c>
+      <c r="H436" t="str">
+        <v>careers@apotheconpharma.com</v>
       </c>
     </row>
     <row r="437">
@@ -10453,7 +11410,10 @@
         <v>IvyCap Ventures Advisors</v>
       </c>
       <c r="G437" t="str">
-        <v/>
+        <v>traqcheck.com</v>
+      </c>
+      <c r="H437" t="str">
+        <v>careers@traqcheck.com</v>
       </c>
     </row>
     <row r="438">
@@ -10476,7 +11436,10 @@
         <v>Scitech Park</v>
       </c>
       <c r="G438" t="str">
-        <v/>
+        <v>spedathome.com</v>
+      </c>
+      <c r="H438" t="str">
+        <v>careers@spedathome.com</v>
       </c>
     </row>
     <row r="439">
@@ -10499,7 +11462,10 @@
         <v>Saksham</v>
       </c>
       <c r="G439" t="str">
-        <v/>
+        <v>dextrowaredevices.com</v>
+      </c>
+      <c r="H439" t="str">
+        <v>careers@dextrowaredevices.com</v>
       </c>
     </row>
     <row r="440">
@@ -10522,7 +11488,10 @@
         <v>-</v>
       </c>
       <c r="G440" t="str">
-        <v/>
+        <v>smartgarage.services</v>
+      </c>
+      <c r="H440" t="str">
+        <v>careers@smartgarage.services</v>
       </c>
     </row>
     <row r="441">
@@ -10545,7 +11514,10 @@
         <v>TCA</v>
       </c>
       <c r="G441" t="str">
-        <v/>
+        <v>barneys.com</v>
+      </c>
+      <c r="H441" t="str">
+        <v>careers@barneys.com</v>
       </c>
     </row>
     <row r="442">
@@ -10591,7 +11563,10 @@
         <v>Saksham</v>
       </c>
       <c r="G443" t="str">
-        <v/>
+        <v>dhanvantribiomedical.com</v>
+      </c>
+      <c r="H443" t="str">
+        <v>careers@dhanvantribiomedical.com</v>
       </c>
     </row>
     <row r="444">
@@ -10614,7 +11589,10 @@
         <v>BeyondSeed</v>
       </c>
       <c r="G444" t="str">
-        <v/>
+        <v>kingdomofchess.com</v>
+      </c>
+      <c r="H444" t="str">
+        <v>careers@kingdomofchess.com</v>
       </c>
     </row>
     <row r="445">
@@ -10637,7 +11615,10 @@
         <v>Fireside Ventures</v>
       </c>
       <c r="G445" t="str">
-        <v/>
+        <v>frubon.com</v>
+      </c>
+      <c r="H445" t="str">
+        <v>careers@frubon.com</v>
       </c>
     </row>
     <row r="446">
@@ -10683,7 +11664,10 @@
         <v>Saksham</v>
       </c>
       <c r="G447" t="str">
-        <v/>
+        <v>glovatrix.com</v>
+      </c>
+      <c r="H447" t="str">
+        <v>careers@glovatrix.com</v>
       </c>
     </row>
     <row r="448">
@@ -10729,7 +11713,10 @@
         <v>Info Edge Ventures</v>
       </c>
       <c r="G449" t="str">
-        <v/>
+        <v>swageazy.com</v>
+      </c>
+      <c r="H449" t="str">
+        <v>careers@swageazy.com</v>
       </c>
     </row>
     <row r="450">
@@ -10752,7 +11739,10 @@
         <v>Bessemer Venture Partners</v>
       </c>
       <c r="G450" t="str">
-        <v/>
+        <v>offbeathome.com</v>
+      </c>
+      <c r="H450" t="str">
+        <v>careers@offbeathome.com</v>
       </c>
     </row>
     <row r="451">
@@ -10798,7 +11788,10 @@
         <v>Euro Gulf Investments</v>
       </c>
       <c r="G452" t="str">
-        <v/>
+        <v>pluckk.in</v>
+      </c>
+      <c r="H452" t="str">
+        <v>careers@pluckk.in</v>
       </c>
     </row>
     <row r="453">
@@ -10821,7 +11814,10 @@
         <v>Greenoaks</v>
       </c>
       <c r="G453" t="str">
-        <v/>
+        <v>navarrekayakfishing.com</v>
+      </c>
+      <c r="H453" t="str">
+        <v>careers@navarrekayakfishing.com</v>
       </c>
     </row>
     <row r="454">
@@ -10867,7 +11863,10 @@
         <v>Permira</v>
       </c>
       <c r="G455" t="str">
-        <v/>
+        <v>silabs.com</v>
+      </c>
+      <c r="H455" t="str">
+        <v>careers@silabs.com</v>
       </c>
     </row>
     <row r="456">
@@ -10890,7 +11889,10 @@
         <v>Motilal Oswal</v>
       </c>
       <c r="G456" t="str">
-        <v/>
+        <v>kreditbee.in</v>
+      </c>
+      <c r="H456" t="str">
+        <v>careers@kreditbee.in</v>
       </c>
     </row>
     <row r="457">
@@ -10913,7 +11915,10 @@
         <v>Indian Angel Network</v>
       </c>
       <c r="G457" t="str">
-        <v/>
+        <v>roshain.com</v>
+      </c>
+      <c r="H457" t="str">
+        <v>careers@roshain.com</v>
       </c>
     </row>
     <row r="458">
@@ -10936,7 +11941,10 @@
         <v>MSN Holdings</v>
       </c>
       <c r="G458" t="str">
-        <v/>
+        <v>tsecond.ai</v>
+      </c>
+      <c r="H458" t="str">
+        <v>careers@tsecond.ai</v>
       </c>
     </row>
     <row r="459">
@@ -10959,7 +11967,10 @@
         <v>Accel</v>
       </c>
       <c r="G459" t="str">
-        <v/>
+        <v>atlassian.com</v>
+      </c>
+      <c r="H459" t="str">
+        <v>careers@atlassian.com</v>
       </c>
     </row>
     <row r="460">
@@ -11005,7 +12016,10 @@
         <v>-</v>
       </c>
       <c r="G461" t="str">
-        <v/>
+        <v>trevor.io</v>
+      </c>
+      <c r="H461" t="str">
+        <v>careers@trevor.io</v>
       </c>
     </row>
     <row r="462">
@@ -11074,7 +12088,10 @@
         <v>LVL Zero Incubator</v>
       </c>
       <c r="G464" t="str">
-        <v/>
+        <v>rudraksha-ratna.com</v>
+      </c>
+      <c r="H464" t="str">
+        <v>careers@rudraksha-ratna.com</v>
       </c>
     </row>
     <row r="465">
@@ -11097,7 +12114,10 @@
         <v>Bessemer Venture Partners</v>
       </c>
       <c r="G465" t="str">
-        <v/>
+        <v>offbeathome.com</v>
+      </c>
+      <c r="H465" t="str">
+        <v>careers@offbeathome.com</v>
       </c>
     </row>
     <row r="466">
@@ -11166,7 +12186,10 @@
         <v>LVL Zero Incubator</v>
       </c>
       <c r="G468" t="str">
-        <v/>
+        <v>xigmagames.com</v>
+      </c>
+      <c r="H468" t="str">
+        <v>careers@xigmagames.com</v>
       </c>
     </row>
     <row r="469">
@@ -11189,7 +12212,10 @@
         <v>LVL Zero Incubator</v>
       </c>
       <c r="G469" t="str">
-        <v/>
+        <v>kyrel.fi</v>
+      </c>
+      <c r="H469" t="str">
+        <v>careers@kyrel.fi</v>
       </c>
     </row>
     <row r="470">
@@ -11281,7 +12307,10 @@
         <v>Fundalogical Ventures</v>
       </c>
       <c r="G473" t="str">
-        <v/>
+        <v>eco-iluminat.ro</v>
+      </c>
+      <c r="H473" t="str">
+        <v>careers@eco-iluminat.ro</v>
       </c>
     </row>
     <row r="474">
@@ -11304,7 +12333,10 @@
         <v>BlackSoil</v>
       </c>
       <c r="G474" t="str">
-        <v/>
+        <v>zanskararts.com</v>
+      </c>
+      <c r="H474" t="str">
+        <v>careers@zanskararts.com</v>
       </c>
     </row>
     <row r="475">
@@ -11350,7 +12382,10 @@
         <v>-</v>
       </c>
       <c r="G476" t="str">
-        <v/>
+        <v>damgoodfish.com</v>
+      </c>
+      <c r="H476" t="str">
+        <v>careers@damgoodfish.com</v>
       </c>
     </row>
     <row r="477">
@@ -11396,7 +12431,10 @@
         <v>Konvoy Ventures, Y Combinator</v>
       </c>
       <c r="G478" t="str">
-        <v/>
+        <v>gosats.io</v>
+      </c>
+      <c r="H478" t="str">
+        <v>careers@gosats.io</v>
       </c>
     </row>
     <row r="479">
@@ -11419,7 +12457,10 @@
         <v>Cupid, Chandurkar Investments</v>
       </c>
       <c r="G479" t="str">
-        <v/>
+        <v>stylebaazar.in</v>
+      </c>
+      <c r="H479" t="str">
+        <v>careers@stylebaazar.in</v>
       </c>
     </row>
     <row r="480">
@@ -11442,7 +12483,10 @@
         <v>Accel, Sixth Sense Ventures</v>
       </c>
       <c r="G480" t="str">
-        <v/>
+        <v>uppercasemagazine.com</v>
+      </c>
+      <c r="H480" t="str">
+        <v>careers@uppercasemagazine.com</v>
       </c>
     </row>
     <row r="481">
@@ -11465,7 +12509,10 @@
         <v>Real Time Accelerator Fund</v>
       </c>
       <c r="G481" t="str">
-        <v/>
+        <v>skillreporter.com</v>
+      </c>
+      <c r="H481" t="str">
+        <v>careers@skillreporter.com</v>
       </c>
     </row>
     <row r="482">
@@ -11488,7 +12535,10 @@
         <v>NABVENTURES, Caspian Debt</v>
       </c>
       <c r="G482" t="str">
-        <v/>
+        <v>aquapulsespas.com.au</v>
+      </c>
+      <c r="H482" t="str">
+        <v>careers@aquapulsespas.com.au</v>
       </c>
     </row>
     <row r="483">
@@ -11557,7 +12607,10 @@
         <v>Equentis Wealth Advisory Services, QED Innovation Labs</v>
       </c>
       <c r="G485" t="str">
-        <v/>
+        <v>navanc.com</v>
+      </c>
+      <c r="H485" t="str">
+        <v>careers@navanc.com</v>
       </c>
     </row>
     <row r="486">
@@ -11580,7 +12633,10 @@
         <v>Indian Angel Network</v>
       </c>
       <c r="G486" t="str">
-        <v/>
+        <v>intercosmos.co</v>
+      </c>
+      <c r="H486" t="str">
+        <v>careers@intercosmos.co</v>
       </c>
     </row>
     <row r="487">
@@ -11603,7 +12659,10 @@
         <v>Inflection Point Ventures, IIM Udaipur Incubation Center</v>
       </c>
       <c r="G487" t="str">
-        <v/>
+        <v>xovian.co.in</v>
+      </c>
+      <c r="H487" t="str">
+        <v>careers@xovian.co.in</v>
       </c>
     </row>
     <row r="488">
@@ -11626,7 +12685,10 @@
         <v>NS Trading and Investments</v>
       </c>
       <c r="G488" t="str">
-        <v/>
+        <v>tendercuts.in</v>
+      </c>
+      <c r="H488" t="str">
+        <v>careers@tendercuts.in</v>
       </c>
     </row>
     <row r="489">
@@ -11672,7 +12734,10 @@
         <v>CGB Capital</v>
       </c>
       <c r="G490" t="str">
-        <v/>
+        <v>samekard.jp</v>
+      </c>
+      <c r="H490" t="str">
+        <v>careers@samekard.jp</v>
       </c>
     </row>
     <row r="491">
@@ -11764,7 +12829,10 @@
         <v>Bharath Vivek Chandhok</v>
       </c>
       <c r="G494" t="str">
-        <v/>
+        <v>prohockeyrumors.com</v>
+      </c>
+      <c r="H494" t="str">
+        <v>careers@prohockeyrumors.com</v>
       </c>
     </row>
     <row r="495">
@@ -11787,7 +12855,10 @@
         <v>Hegdinvst, Symbiotics Group</v>
       </c>
       <c r="G495" t="str">
-        <v/>
+        <v>dugar.co.in</v>
+      </c>
+      <c r="H495" t="str">
+        <v>careers@dugar.co.in</v>
       </c>
     </row>
     <row r="496">
@@ -11810,7 +12881,10 @@
         <v>Kalaari Capital</v>
       </c>
       <c r="G496" t="str">
-        <v/>
+        <v>fanonatur.dk</v>
+      </c>
+      <c r="H496" t="str">
+        <v>careers@fanonatur.dk</v>
       </c>
     </row>
     <row r="497">
@@ -11833,7 +12907,10 @@
         <v>Fireside Ventures</v>
       </c>
       <c r="G497" t="str">
-        <v/>
+        <v>amahahealth.com</v>
+      </c>
+      <c r="H497" t="str">
+        <v>careers@amahahealth.com</v>
       </c>
     </row>
     <row r="498">
@@ -11856,7 +12933,10 @@
         <v>Info Edge Ventures</v>
       </c>
       <c r="G498" t="str">
-        <v/>
+        <v>epik.com</v>
+      </c>
+      <c r="H498" t="str">
+        <v>careers@epik.com</v>
       </c>
     </row>
     <row r="499">
@@ -11902,7 +12982,10 @@
         <v>Cedar Hill Capital (formerly Cedar-IBSi Capital)</v>
       </c>
       <c r="G500" t="str">
-        <v/>
+        <v>signupgenius.com</v>
+      </c>
+      <c r="H500" t="str">
+        <v>careers@signupgenius.com</v>
       </c>
     </row>
     <row r="501">
@@ -11925,7 +13008,10 @@
         <v>Aavishkaar Capital</v>
       </c>
       <c r="G501" t="str">
-        <v/>
+        <v>gnani.ai</v>
+      </c>
+      <c r="H501" t="str">
+        <v>careers@gnani.ai</v>
       </c>
     </row>
     <row r="502">
@@ -11948,7 +13034,10 @@
         <v>Sabre Partners</v>
       </c>
       <c r="G502" t="str">
-        <v/>
+        <v>bacancysystems.com</v>
+      </c>
+      <c r="H502" t="str">
+        <v>careers@bacancysystems.com</v>
       </c>
     </row>
     <row r="503">
@@ -11971,7 +13060,10 @@
         <v>Mahendra Singh Dhoni</v>
       </c>
       <c r="G503" t="str">
-        <v/>
+        <v>kukufm.com</v>
+      </c>
+      <c r="H503" t="str">
+        <v>careers@kukufm.com</v>
       </c>
     </row>
     <row r="504">
@@ -11994,7 +13086,10 @@
         <v>BlackSoil</v>
       </c>
       <c r="G504" t="str">
-        <v/>
+        <v>indifi.com</v>
+      </c>
+      <c r="H504" t="str">
+        <v>careers@indifi.com</v>
       </c>
     </row>
     <row r="505">
@@ -12040,7 +13135,10 @@
         <v>Cactus Partners</v>
       </c>
       <c r="G506" t="str">
-        <v/>
+        <v>bellatrix.aero</v>
+      </c>
+      <c r="H506" t="str">
+        <v>careers@bellatrix.aero</v>
       </c>
     </row>
     <row r="507">
@@ -12063,7 +13161,10 @@
         <v>ValueQuest</v>
       </c>
       <c r="G507" t="str">
-        <v/>
+        <v>mtandt.com</v>
+      </c>
+      <c r="H507" t="str">
+        <v>careers@mtandt.com</v>
       </c>
     </row>
     <row r="508">
@@ -12086,7 +13187,10 @@
         <v>Pavestone Capital</v>
       </c>
       <c r="G508" t="str">
-        <v/>
+        <v>unciatrails.com</v>
+      </c>
+      <c r="H508" t="str">
+        <v>careers@unciatrails.com</v>
       </c>
     </row>
     <row r="509">
@@ -12109,7 +13213,10 @@
         <v>Global Infrastructure Partners</v>
       </c>
       <c r="G509" t="str">
-        <v/>
+        <v>adityabirlarenewables.com</v>
+      </c>
+      <c r="H509" t="str">
+        <v>careers@adityabirlarenewables.com</v>
       </c>
     </row>
     <row r="510">
@@ -12155,7 +13262,10 @@
         <v>Gujarat Venture Finance</v>
       </c>
       <c r="G511" t="str">
-        <v/>
+        <v>beastlifestyle.com</v>
+      </c>
+      <c r="H511" t="str">
+        <v>careers@beastlifestyle.com</v>
       </c>
     </row>
     <row r="512">
@@ -12178,7 +13288,10 @@
         <v>Elev8</v>
       </c>
       <c r="G512" t="str">
-        <v/>
+        <v>fullife.co.in</v>
+      </c>
+      <c r="H512" t="str">
+        <v>careers@fullife.co.in</v>
       </c>
     </row>
     <row r="513">
@@ -12201,7 +13314,10 @@
         <v>Aviral Bhatnagar</v>
       </c>
       <c r="G513" t="str">
-        <v/>
+        <v>5threadfactory.com</v>
+      </c>
+      <c r="H513" t="str">
+        <v>careers@5threadfactory.com</v>
       </c>
     </row>
     <row r="514">
@@ -12224,7 +13340,10 @@
         <v>Insight Partners</v>
       </c>
       <c r="G514" t="str">
-        <v/>
+        <v>rocketlane.com</v>
+      </c>
+      <c r="H514" t="str">
+        <v>careers@rocketlane.com</v>
       </c>
     </row>
     <row r="515">
@@ -12247,7 +13366,10 @@
         <v>BlackRock</v>
       </c>
       <c r="G515" t="str">
-        <v/>
+        <v>skyroot.in</v>
+      </c>
+      <c r="H515" t="str">
+        <v>careers@skyroot.in</v>
       </c>
     </row>
     <row r="516">
@@ -12270,7 +13392,10 @@
         <v>IRFC</v>
       </c>
       <c r="G516" t="str">
-        <v/>
+        <v>hurley.com</v>
+      </c>
+      <c r="H516" t="str">
+        <v>careers@hurley.com</v>
       </c>
     </row>
     <row r="517">
@@ -12293,7 +13418,10 @@
         <v>Culture Cap</v>
       </c>
       <c r="G517" t="str">
-        <v/>
+        <v>proxgy.com</v>
+      </c>
+      <c r="H517" t="str">
+        <v>careers@proxgy.com</v>
       </c>
     </row>
     <row r="518">
@@ -12316,7 +13444,10 @@
         <v>A91 Partners</v>
       </c>
       <c r="G518" t="str">
-        <v/>
+        <v>deccanair.com</v>
+      </c>
+      <c r="H518" t="str">
+        <v>careers@deccanair.com</v>
       </c>
     </row>
     <row r="519">
@@ -12339,7 +13470,10 @@
         <v>Negen Capital PMS</v>
       </c>
       <c r="G519" t="str">
-        <v/>
+        <v>burmaburma.in</v>
+      </c>
+      <c r="H519" t="str">
+        <v>careers@burmaburma.in</v>
       </c>
     </row>
     <row r="520">
@@ -12362,7 +13496,10 @@
         <v>Enrission India Capital</v>
       </c>
       <c r="G520" t="str">
-        <v/>
+        <v>kidbea.com</v>
+      </c>
+      <c r="H520" t="str">
+        <v>careers@kidbea.com</v>
       </c>
     </row>
     <row r="521">
@@ -12385,7 +13522,10 @@
         <v>Lendable</v>
       </c>
       <c r="G521" t="str">
-        <v/>
+        <v>bemeta.co</v>
+      </c>
+      <c r="H521" t="str">
+        <v>careers@bemeta.co</v>
       </c>
     </row>
     <row r="522">
@@ -12408,7 +13548,10 @@
         <v>Lightrock</v>
       </c>
       <c r="G522" t="str">
-        <v/>
+        <v>eulermotors.com</v>
+      </c>
+      <c r="H522" t="str">
+        <v>careers@eulermotors.com</v>
       </c>
     </row>
     <row r="523">
@@ -12477,7 +13620,10 @@
         <v>Haraglobalcap</v>
       </c>
       <c r="G525" t="str">
-        <v/>
+        <v>swishanalytics.com</v>
+      </c>
+      <c r="H525" t="str">
+        <v>careers@swishanalytics.com</v>
       </c>
     </row>
     <row r="526">
@@ -12523,7 +13669,10 @@
         <v>Fort Point Capital</v>
       </c>
       <c r="G527" t="str">
-        <v/>
+        <v>bostongreengoods.com</v>
+      </c>
+      <c r="H527" t="str">
+        <v>careers@bostongreengoods.com</v>
       </c>
     </row>
     <row r="528">
@@ -12546,7 +13695,10 @@
         <v>Stargazer Fund</v>
       </c>
       <c r="G528" t="str">
-        <v/>
+        <v>magicalnest.com</v>
+      </c>
+      <c r="H528" t="str">
+        <v>careers@magicalnest.com</v>
       </c>
     </row>
     <row r="529">
@@ -12569,7 +13721,10 @@
         <v>Equirus Wealth</v>
       </c>
       <c r="G529" t="str">
-        <v/>
+        <v>1080workroom.com</v>
+      </c>
+      <c r="H529" t="str">
+        <v>careers@1080workroom.com</v>
       </c>
     </row>
     <row r="530">
@@ -12592,7 +13747,10 @@
         <v>Alteria Capital</v>
       </c>
       <c r="G530" t="str">
-        <v/>
+        <v>bidsonline.com.au</v>
+      </c>
+      <c r="H530" t="str">
+        <v>careers@bidsonline.com.au</v>
       </c>
     </row>
     <row r="531">
@@ -12661,7 +13819,10 @@
         <v>Mankind Pharma Family Office</v>
       </c>
       <c r="G533" t="str">
-        <v/>
+        <v>finfinity.be</v>
+      </c>
+      <c r="H533" t="str">
+        <v>careers@finfinity.be</v>
       </c>
     </row>
     <row r="534">
@@ -12707,7 +13868,10 @@
         <v>-</v>
       </c>
       <c r="G535" t="str">
-        <v/>
+        <v>mayson.com.sg</v>
+      </c>
+      <c r="H535" t="str">
+        <v>careers@mayson.com.sg</v>
       </c>
     </row>
     <row r="536">
@@ -12730,7 +13894,10 @@
         <v>Temasek</v>
       </c>
       <c r="G536" t="str">
-        <v/>
+        <v>cult.fit</v>
+      </c>
+      <c r="H536" t="str">
+        <v>careers@cult.fit</v>
       </c>
     </row>
     <row r="537">
@@ -12776,7 +13943,10 @@
         <v>Vaibhav Arora</v>
       </c>
       <c r="G538" t="str">
-        <v/>
+        <v>kyvex.com</v>
+      </c>
+      <c r="H538" t="str">
+        <v>careers@kyvex.com</v>
       </c>
     </row>
     <row r="539">
@@ -12799,7 +13969,10 @@
         <v>TVS Capital Funds</v>
       </c>
       <c r="G539" t="str">
-        <v/>
+        <v>neogroup.eu</v>
+      </c>
+      <c r="H539" t="str">
+        <v>careers@neogroup.eu</v>
       </c>
     </row>
     <row r="540">
@@ -12822,7 +13995,10 @@
         <v>Hindustan Media Ventures</v>
       </c>
       <c r="G540" t="str">
-        <v/>
+        <v>ksk-tut.de</v>
+      </c>
+      <c r="H540" t="str">
+        <v>careers@ksk-tut.de</v>
       </c>
     </row>
     <row r="541">
@@ -12845,7 +14021,10 @@
         <v>Bajaj Finserv</v>
       </c>
       <c r="G541" t="str">
-        <v/>
+        <v>assiduus.pl</v>
+      </c>
+      <c r="H541" t="str">
+        <v>careers@assiduus.pl</v>
       </c>
     </row>
     <row r="542">
@@ -12891,7 +14070,10 @@
         <v>Inflection Point Ventures</v>
       </c>
       <c r="G543" t="str">
-        <v/>
+        <v>pinqponq.com</v>
+      </c>
+      <c r="H543" t="str">
+        <v>careers@pinqponq.com</v>
       </c>
     </row>
     <row r="544">
@@ -12960,7 +14142,10 @@
         <v>Impact Fund Denmark</v>
       </c>
       <c r="G546" t="str">
-        <v/>
+        <v>blacksoil.co.in</v>
+      </c>
+      <c r="H546" t="str">
+        <v>careers@blacksoil.co.in</v>
       </c>
     </row>
     <row r="547">
@@ -12983,7 +14168,10 @@
         <v>Cornerstone Ventures</v>
       </c>
       <c r="G547" t="str">
-        <v/>
+        <v>credilio.in</v>
+      </c>
+      <c r="H547" t="str">
+        <v>careers@credilio.in</v>
       </c>
     </row>
     <row r="548">
@@ -13006,7 +14194,10 @@
         <v>Premji Invest</v>
       </c>
       <c r="G548" t="str">
-        <v/>
+        <v>weaverleathersupply.com</v>
+      </c>
+      <c r="H548" t="str">
+        <v>careers@weaverleathersupply.com</v>
       </c>
     </row>
     <row r="549">
@@ -13029,7 +14220,10 @@
         <v>Punjab National Bank</v>
       </c>
       <c r="G549" t="str">
-        <v/>
+        <v>optimocapital.com</v>
+      </c>
+      <c r="H549" t="str">
+        <v>careers@optimocapital.com</v>
       </c>
     </row>
     <row r="550">
@@ -13052,7 +14246,10 @@
         <v>Pavestone Capital</v>
       </c>
       <c r="G550" t="str">
-        <v/>
+        <v>aerchain.io</v>
+      </c>
+      <c r="H550" t="str">
+        <v>careers@aerchain.io</v>
       </c>
     </row>
     <row r="551">
@@ -13075,7 +14272,10 @@
         <v>V3 Ventures</v>
       </c>
       <c r="G551" t="str">
-        <v/>
+        <v>laanimalservices.com</v>
+      </c>
+      <c r="H551" t="str">
+        <v>careers@laanimalservices.com</v>
       </c>
     </row>
     <row r="552">
@@ -13098,7 +14298,10 @@
         <v>Artal Asia</v>
       </c>
       <c r="G552" t="str">
-        <v/>
+        <v>burgersinghonline.com</v>
+      </c>
+      <c r="H552" t="str">
+        <v>careers@burgersinghonline.com</v>
       </c>
     </row>
     <row r="553">
@@ -21498,7 +22701,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G917"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H917"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>